<commit_message>
Lauf 2026-09-13 11:15 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1544,48 +1544,52 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="n">
-        <v>72</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Exclusive Associates</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>5</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Unterhaching, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1605,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1631,7 +1635,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1642,21 +1646,21 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
@@ -1666,7 +1670,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1677,31 +1681,33 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>Feuersbach, Siegen</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2</v>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
@@ -1710,7 +1716,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1721,28 +1727,28 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1754,7 +1760,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1765,7 +1771,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1787,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1798,7 +1804,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1809,7 +1815,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1825,12 +1831,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1842,7 +1848,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1853,7 +1859,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1875,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1886,7 +1892,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1897,33 +1903,31 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
@@ -1932,7 +1936,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1943,33 +1947,31 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
@@ -1978,7 +1980,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1989,7 +1991,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2007,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2016,11 +2018,7 @@
       <c r="F34" t="n">
         <v>6</v>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2039,7 +2037,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2050,17 +2048,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2085,7 +2083,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2096,17 +2094,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2114,7 +2112,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2135,40 +2133,42 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>6</v>
+      </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2179,32 +2179,38 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+          <t>Braunsfeld, Köln</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>6</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2223,40 +2229,40 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2267,7 +2273,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
@@ -2278,17 +2284,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2311,7 +2317,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2322,17 +2328,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2355,7 +2361,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2366,17 +2372,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2388,7 +2394,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2399,7 +2405,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2421,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2432,7 +2438,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2443,7 +2449,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2465,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2476,7 +2482,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2487,7 +2493,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2498,17 +2504,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2520,7 +2526,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2531,7 +2537,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2542,17 +2548,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2564,7 +2570,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2575,28 +2581,28 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2619,28 +2625,28 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2652,7 +2658,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2663,7 +2669,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2690,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2696,7 +2702,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2707,23 +2713,23 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2740,7 +2746,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2751,28 +2757,28 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2784,7 +2790,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2795,7 +2801,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2806,12 +2812,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2839,7 +2845,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2850,12 +2856,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2872,7 +2878,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2883,7 +2889,7 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -2894,12 +2900,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2916,7 +2922,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2927,7 +2933,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2949,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2960,7 +2966,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2971,40 +2977,40 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3015,7 +3021,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
@@ -3026,29 +3032,29 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3059,28 +3065,28 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -3092,7 +3098,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3103,7 +3109,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3130,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -3147,33 +3153,31 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>6</v>
-      </c>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3193,7 +3197,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3208,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3214,7 +3218,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -3239,31 +3243,33 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>6</v>
+      </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
@@ -3283,7 +3289,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3294,17 +3300,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -3316,7 +3322,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3327,7 +3333,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3338,12 +3344,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3352,11 +3358,7 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3364,7 +3366,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3375,7 +3377,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3386,24 +3388,28 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3419,7 +3425,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3441,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3452,7 +3458,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3463,7 +3469,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3485,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3496,7 +3502,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3507,46 +3513,40 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F68" t="n">
-        <v>6</v>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3557,7 +3557,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3607,7 +3607,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3618,29 +3618,35 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>6</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3651,7 +3657,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3662,29 +3668,29 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3695,28 +3701,28 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -3728,7 +3734,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3739,7 +3745,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
@@ -3750,17 +3756,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3772,7 +3778,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3783,7 +3789,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3794,25 +3800,21 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3831,7 +3833,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3842,12 +3844,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3858,7 +3860,7 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3868,7 +3870,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3879,7 +3881,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3897,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3916,7 +3918,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3938,21 +3940,25 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3960,7 +3966,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3971,76 +3977,72 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="n">
+        <v>51</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>WirWinzer</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Altstadt-Lehel, München</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>yoursquares GmbH</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>Tiergarten, Berlin</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr"/>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4052,7 +4054,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4063,7 +4065,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4081,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4088,11 +4090,7 @@
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4100,7 +4098,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4111,7 +4109,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -4122,29 +4120,33 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4155,7 +4157,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
         </is>
       </c>
     </row>
@@ -4166,35 +4168,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F82" t="n">
-        <v>6</v>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4205,36 +4201,46 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>6</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4245,51 +4251,47 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="n">
+        <v>49</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ABOUT YOU</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
           <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>ABOUT YOU</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr"/>
-      <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" s="2" t="inlineStr"/>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K84" s="2" t="inlineStr"/>
-      <c r="L84" s="2" t="inlineStr">
-        <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4300,29 +4302,25 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4333,7 +4331,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4354,7 +4352,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4366,7 +4364,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4377,7 +4375,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4388,17 +4386,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4410,7 +4408,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4421,7 +4419,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4432,15 +4430,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -4450,7 +4452,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4461,51 +4463,47 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="n">
+        <v>49</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Coty</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
           <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>Coty</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>Skincare Merchandising Intern</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr"/>
-      <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" s="2" t="inlineStr"/>
-      <c r="H89" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I89" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="J89" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K89" s="2" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr">
-        <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4516,19 +4514,15 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -4538,7 +4532,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4549,7 +4543,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4560,17 +4554,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4582,7 +4576,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4593,7 +4587,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4604,17 +4598,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4626,7 +4620,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4637,7 +4631,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4648,24 +4642,24 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -4681,7 +4675,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4697,12 +4691,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4714,7 +4708,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4725,55 +4719,51 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="n">
+        <v>49</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2 Standorte</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
           <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B95" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>Mars</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>DEU-Bayern-Unterhaching</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" s="2" t="inlineStr"/>
-      <c r="H95" s="2" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I95" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="J95" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K95" s="2" t="inlineStr"/>
-      <c r="L95" s="2" t="inlineStr">
-        <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4784,29 +4774,29 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4817,7 +4807,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4828,17 +4818,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4861,7 +4851,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4867,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4905,7 +4895,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4911,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4949,7 +4939,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4960,17 +4950,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4993,7 +4983,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -5004,17 +4994,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5026,7 +5016,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5037,28 +5027,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5070,7 +5060,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5081,28 +5071,28 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5114,7 +5104,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5125,7 +5115,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5136,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5169,28 +5159,28 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr"/>
       <c r="B105" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5202,7 +5192,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5213,7 +5203,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5224,17 +5214,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5246,7 +5236,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5257,7 +5247,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5268,17 +5258,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5290,7 +5280,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5301,7 +5291,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5307,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5345,7 +5335,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5361,12 +5351,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5389,7 +5379,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5405,7 +5395,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5433,7 +5423,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5444,17 +5434,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -5477,7 +5467,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5488,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5521,12 +5511,56 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr"/>
+      <c r="B113" t="n">
+        <v>45</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L112"/>
+  <autoFilter ref="A1:L113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5593,7 +5627,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5668,7 +5702,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -5693,7 +5727,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C6" t="n">
         <v>89</v>
@@ -5751,7 +5785,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" t="n">
         <v>87</v>
@@ -5776,7 +5810,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5801,7 +5835,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5826,7 +5860,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5859,7 +5893,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5892,7 +5926,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5917,7 +5951,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5942,7 +5976,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -5967,7 +6001,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5992,7 +6026,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6067,7 +6101,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C20" t="n">
         <v>83</v>
@@ -6125,7 +6159,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C22" t="n">
         <v>79</v>
@@ -6200,7 +6234,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6225,7 +6259,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6250,7 +6284,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6300,7 +6334,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6325,7 +6359,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6383,7 +6417,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6408,7 +6442,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6483,7 +6517,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6583,7 +6617,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6608,7 +6642,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6633,7 +6667,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6658,7 +6692,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -6691,7 +6725,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -6716,7 +6750,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6766,7 +6800,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6799,7 +6833,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6824,7 +6858,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6874,7 +6908,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C51" t="n">
         <v>54</v>
@@ -6899,7 +6933,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6924,7 +6958,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -7074,7 +7108,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -7099,7 +7133,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -7174,7 +7208,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7199,7 +7233,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7224,7 +7258,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7274,7 +7308,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7299,7 +7333,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -7324,7 +7358,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7349,7 +7383,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
@@ -7374,7 +7408,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7824,7 +7858,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C89" t="n">
         <v>46</v>
@@ -7874,7 +7908,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C91" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-14 11:56 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1596,25 +1596,25 @@
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1635,7 +1635,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1681,7 +1681,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1692,21 +1692,21 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1727,31 +1727,33 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>Feuersbach, Siegen</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2</v>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
@@ -1760,7 +1762,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1771,28 +1773,28 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -1804,7 +1806,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1815,7 +1817,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1833,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1848,7 +1850,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1859,7 +1861,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1882,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1892,7 +1894,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1903,7 +1905,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -2144,23 +2146,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>6</v>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2179,46 +2185,40 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>6</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2229,40 +2229,40 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2273,7 +2273,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2317,7 +2317,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2328,17 +2328,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2361,7 +2361,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2372,17 +2372,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2405,7 +2405,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2449,7 +2449,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2493,7 +2493,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2537,7 +2537,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2548,17 +2548,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2581,7 +2581,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2625,28 +2625,28 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2669,28 +2669,28 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2713,23 +2713,23 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2757,14 +2757,14 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2773,12 +2773,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2801,7 +2801,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -2812,12 +2812,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2845,7 +2845,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
@@ -2856,12 +2856,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2889,40 +2889,40 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2933,28 +2933,28 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2977,28 +2977,28 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3021,35 +3021,35 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3065,31 +3065,33 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>6</v>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3098,7 +3100,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3109,31 +3111,33 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>6</v>
+      </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
@@ -3153,28 +3157,28 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -3197,33 +3201,31 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F61" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
@@ -3232,7 +3234,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3243,34 +3245,36 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F62" t="n">
-        <v>6</v>
-      </c>
-      <c r="G62" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3289,7 +3293,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3300,24 +3304,24 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3333,7 +3337,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3344,29 +3348,29 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3377,7 +3381,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
@@ -3388,33 +3392,29 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3425,40 +3425,46 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>6</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3469,40 +3475,46 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>6</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3513,40 +3525,40 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3557,7 +3569,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3568,27 +3580,21 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F69" t="n">
-        <v>6</v>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3596,7 +3602,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3607,7 +3613,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3618,27 +3624,21 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F70" t="n">
-        <v>6</v>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3657,40 +3657,40 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3701,28 +3701,28 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3745,7 +3745,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3756,21 +3756,25 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3778,7 +3782,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3789,7 +3793,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3800,21 +3804,25 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3822,7 +3830,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3833,7 +3841,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3844,12 +3852,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3860,7 +3868,7 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3870,7 +3878,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3881,7 +3889,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3892,25 +3900,21 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3918,7 +3922,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3929,7 +3933,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3940,25 +3944,21 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3977,28 +3977,28 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4021,32 +4021,36 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4054,7 +4058,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4065,7 +4069,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
         </is>
       </c>
     </row>
@@ -4076,29 +4080,29 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4109,7 +4113,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4120,20 +4124,22 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr"/>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>6</v>
+      </c>
       <c r="G81" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -4146,7 +4152,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4157,30 +4163,26 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
@@ -4190,7 +4192,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4201,46 +4203,36 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F83" t="n">
-        <v>6</v>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4251,7 +4243,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4262,25 +4254,29 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr"/>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Hannover, Region Hannover (Kreis)</t>
+        </is>
+      </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4291,7 +4287,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4302,25 +4298,29 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr"/>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Bult, Hannover</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4331,7 +4331,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4342,17 +4342,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
+          <t>Unterbilk, Düsseldorf</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4375,7 +4375,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4386,19 +4386,15 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Bult, Hannover</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
@@ -4408,7 +4404,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4419,7 +4415,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4430,19 +4426,15 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Unterbilk, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -4452,7 +4444,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4463,7 +4455,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4474,15 +4466,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Berlin, Berlin, Germany</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -4492,7 +4488,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4503,7 +4499,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4514,15 +4510,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr"/>
+          <t>Praktikum Category Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Münster, Nordrhein-Westfalen</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4543,7 +4543,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4554,17 +4554,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4587,7 +4587,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4598,29 +4598,29 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4631,7 +4631,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4642,29 +4642,29 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4675,7 +4675,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4730,29 +4730,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4763,7 +4763,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4774,29 +4774,29 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4807,7 +4807,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4818,17 +4818,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4851,7 +4851,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4862,17 +4862,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4895,7 +4895,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4906,17 +4906,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4928,7 +4928,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4939,28 +4939,28 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4983,28 +4983,28 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5027,28 +5027,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5071,28 +5071,28 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5115,28 +5115,28 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5159,28 +5159,28 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr"/>
       <c r="B105" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5203,7 +5203,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5214,17 +5214,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5247,7 +5247,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5258,17 +5258,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5291,7 +5291,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5307,12 +5307,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5335,7 +5335,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5346,12 +5346,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5379,7 +5379,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5390,12 +5390,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5423,144 +5423,12 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr"/>
-      <c r="B111" t="n">
-        <v>45</v>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>prepmymeal GmbH</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr"/>
-      <c r="B112" t="n">
-        <v>45</v>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr"/>
-      <c r="B113" t="n">
-        <v>45</v>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L113"/>
+  <autoFilter ref="A1:L110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5627,7 +5495,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5727,7 +5595,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C6" t="n">
         <v>89</v>
@@ -5785,7 +5653,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
         <v>87</v>
@@ -5810,7 +5678,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5835,7 +5703,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5860,7 +5728,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5893,7 +5761,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5926,7 +5794,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5951,7 +5819,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5976,7 +5844,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6001,7 +5869,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6026,7 +5894,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6051,7 +5919,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -6101,7 +5969,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C20" t="n">
         <v>83</v>
@@ -6159,7 +6027,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C22" t="n">
         <v>79</v>
@@ -6234,7 +6102,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6259,7 +6127,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6284,7 +6152,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6334,7 +6202,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6359,7 +6227,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6417,7 +6285,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6442,7 +6310,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6517,7 +6385,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6617,7 +6485,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6642,7 +6510,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6667,7 +6535,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6692,7 +6560,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -6725,7 +6593,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -6750,7 +6618,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6800,7 +6668,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6833,7 +6701,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6858,7 +6726,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6908,7 +6776,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C51" t="n">
         <v>54</v>
@@ -6933,7 +6801,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6958,7 +6826,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -7108,7 +6976,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -7133,7 +7001,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -7208,7 +7076,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7233,7 +7101,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7258,7 +7126,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7308,7 +7176,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7333,7 +7201,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -7358,7 +7226,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7383,7 +7251,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
@@ -7408,7 +7276,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7858,7 +7726,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C89" t="n">
         <v>46</v>
@@ -7908,7 +7776,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C91" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-15 11:15 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -752,25 +752,25 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -791,7 +791,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -825,12 +825,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -841,7 +841,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -852,31 +852,35 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -887,7 +891,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -903,7 +907,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -922,7 +926,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -933,7 +937,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -949,12 +953,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -968,7 +972,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -979,7 +983,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -990,17 +994,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1014,7 +1018,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1025,7 +1029,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1050,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1071,36 +1075,34 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1119,36 +1121,34 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>6</v>
-      </c>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1169,7 +1169,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1196,7 +1196,11 @@
       <c r="F16" t="n">
         <v>6</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1215,7 +1219,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1226,17 +1230,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1250,7 +1254,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1261,7 +1265,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1272,27 +1276,23 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1311,7 +1311,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1332,13 +1332,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>6</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1357,31 +1361,33 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
@@ -1390,7 +1396,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1401,7 +1407,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1423,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1445,7 +1451,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
@@ -1456,27 +1462,21 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HUGO BOSS</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Metzingen, Reutlingen (Kreis)</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>6</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1495,7 +1495,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
@@ -1506,21 +1506,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>HUGO BOSS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+          <t>Metzingen, Reutlingen (Kreis)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1528,7 +1534,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1539,57 +1545,51 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="n">
+        <v>74</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Miles &amp; More GmbH</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Mars</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Unterhaching, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1600,17 +1600,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1635,32 +1635,32 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1681,7 +1681,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1727,7 +1727,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1738,21 +1738,21 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1773,31 +1773,33 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>Feuersbach, Siegen</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
@@ -1806,7 +1808,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1817,28 +1819,28 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1850,7 +1852,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1861,7 +1863,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1879,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1894,7 +1896,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1905,7 +1907,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1921,12 +1923,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1938,7 +1940,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1949,7 +1951,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1967,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1982,7 +1984,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1993,33 +1995,31 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2039,33 +2039,31 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
@@ -2074,7 +2072,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2085,7 +2083,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2099,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2112,11 +2110,7 @@
       <c r="F36" t="n">
         <v>6</v>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2135,7 +2129,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2146,27 +2140,23 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>6</v>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2185,40 +2175,46 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>6</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2229,32 +2225,38 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
+          <t>Braunsfeld, Köln</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>6</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2273,28 +2275,28 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2317,40 +2319,40 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2361,7 +2363,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
@@ -2372,17 +2374,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2405,7 +2407,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2416,17 +2418,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2438,7 +2440,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2449,7 +2451,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2460,17 +2462,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2482,7 +2484,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2493,7 +2495,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2511,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2526,7 +2528,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2537,7 +2539,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2548,17 +2550,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2570,7 +2572,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2581,7 +2583,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2594,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2614,7 +2616,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2625,28 +2627,28 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2658,7 +2660,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2669,28 +2671,28 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2702,7 +2704,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2713,28 +2715,28 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2746,7 +2748,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2757,14 +2759,14 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2773,12 +2775,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2790,7 +2792,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2801,51 +2803,53 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="n">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Coty</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -2856,12 +2860,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2878,7 +2882,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2889,40 +2893,40 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2933,28 +2937,28 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2966,7 +2970,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2977,28 +2981,28 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3010,7 +3014,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3021,35 +3025,35 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3065,33 +3069,31 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>6</v>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3111,33 +3113,31 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F59" t="n">
-        <v>6</v>
-      </c>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
@@ -3157,31 +3157,33 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>6</v>
+      </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3201,31 +3203,33 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>6</v>
+      </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
@@ -3234,7 +3238,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3245,7 +3249,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3256,12 +3260,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3270,11 +3274,7 @@
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3293,7 +3293,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5595,7 +5595,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C6" t="n">
         <v>89</v>
@@ -5653,7 +5653,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
         <v>87</v>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5703,7 +5703,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5728,7 +5728,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5761,7 +5761,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5794,7 +5794,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5819,7 +5819,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5844,7 +5844,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -5869,7 +5869,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5894,7 +5894,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -5915,18 +5915,18 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -5940,80 +5940,80 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>115</v>
+        <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>40</v>
+        <v>117</v>
       </c>
       <c r="C21" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6023,18 +6023,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -6102,7 +6102,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6127,7 +6127,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6202,7 +6202,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6285,7 +6285,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6310,7 +6310,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6385,7 +6385,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6510,7 +6510,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6535,7 +6535,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6560,7 +6560,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -6593,7 +6593,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -6668,7 +6668,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6701,7 +6701,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6726,7 +6726,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6776,7 +6776,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C51" t="n">
         <v>54</v>
@@ -6801,7 +6801,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6826,7 +6826,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -6976,7 +6976,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -7001,7 +7001,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -7076,7 +7076,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7101,7 +7101,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7126,7 +7126,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7176,7 +7176,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7201,7 +7201,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -7226,7 +7226,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7251,7 +7251,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
@@ -7276,7 +7276,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7726,7 +7726,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C89" t="n">
         <v>46</v>
@@ -7776,7 +7776,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C91" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-16 11:01 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -522,17 +522,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -557,7 +557,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
@@ -752,25 +752,25 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -791,7 +791,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -825,12 +825,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -841,7 +841,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -852,35 +852,31 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -891,7 +887,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -907,7 +903,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -926,7 +922,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -937,7 +933,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -953,12 +949,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -972,7 +968,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -983,7 +979,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -994,17 +990,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1018,7 +1014,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1029,7 +1025,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1046,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1075,34 +1071,36 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1121,34 +1119,36 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>6</v>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1169,7 +1169,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1196,11 +1196,7 @@
       <c r="F16" t="n">
         <v>6</v>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1219,7 +1215,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1230,17 +1226,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1254,7 +1250,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1265,7 +1261,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1276,23 +1272,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1311,7 +1311,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1332,17 +1332,13 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>6</v>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1361,33 +1357,31 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>6</v>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
@@ -1396,7 +1390,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1407,7 +1401,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1417,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1451,7 +1445,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
@@ -1462,21 +1456,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>HUGO BOSS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+          <t>Metzingen, Reutlingen (Kreis)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1495,7 +1495,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1506,27 +1506,21 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HUGO BOSS</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Metzingen, Reutlingen (Kreis)</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1534,7 +1528,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1545,7 +1539,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1556,20 +1550,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>6</v>
+      </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
@@ -1589,7 +1585,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1826,21 +1822,21 @@
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1852,7 +1848,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1863,7 +1859,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1875,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1896,7 +1892,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1907,7 +1903,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1924,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1940,7 +1936,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1951,7 +1947,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1963,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1984,7 +1980,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1995,7 +1991,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2007,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2039,31 +2035,33 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
+          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>6</v>
+      </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
@@ -2072,7 +2070,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2083,7 +2081,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2097,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2129,7 +2127,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2143,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2156,7 +2154,11 @@
       <c r="F37" t="n">
         <v>6</v>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2175,7 +2177,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2186,17 +2188,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2204,7 +2206,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2225,46 +2227,40 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>6</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2275,28 +2271,28 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2319,40 +2315,40 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2363,7 +2359,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2374,17 +2370,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2407,7 +2403,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2418,17 +2414,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2451,7 +2447,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2462,17 +2458,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2484,7 +2480,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2495,7 +2491,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2507,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2528,7 +2524,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2539,7 +2535,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2551,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2572,7 +2568,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2583,7 +2579,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2594,17 +2590,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2616,7 +2612,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2627,7 +2623,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
@@ -2638,17 +2634,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2660,7 +2656,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2671,28 +2667,28 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2715,28 +2711,28 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2748,7 +2744,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2759,28 +2755,28 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2792,7 +2788,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2803,53 +2799,51 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="n">
         <v>59</v>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Coty</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Otto GmbH &amp; Co. KGaA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -2860,12 +2854,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2882,7 +2876,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2893,40 +2887,40 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2937,28 +2931,28 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2970,7 +2964,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2981,28 +2975,28 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3014,7 +3008,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3025,75 +3019,77 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="n">
-        <v>57</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Richemont</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Coty</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>6</v>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3113,31 +3109,33 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>6</v>
+      </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
@@ -3157,33 +3155,31 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>6</v>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3203,33 +3199,31 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F61" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
@@ -3238,7 +3232,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3249,7 +3243,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3260,12 +3254,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3274,7 +3268,11 @@
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3282,7 +3280,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3293,7 +3291,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4118,81 +4116,89 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="n">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>RÖDL</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F81" t="n">
-        <v>6</v>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Richemont</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>High Jewelry Business Development Assistant Intern</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>6</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4203,7 +4209,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4225,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -4232,7 +4238,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4243,7 +4249,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4254,29 +4260,25 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4287,7 +4289,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4310,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4320,7 +4322,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4331,7 +4333,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4342,17 +4344,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4364,7 +4366,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4375,7 +4377,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4386,15 +4388,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
@@ -4404,7 +4410,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4415,7 +4421,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4437,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -4444,7 +4450,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4455,7 +4461,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4466,19 +4472,15 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -4488,7 +4490,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4499,7 +4501,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4510,17 +4512,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4532,7 +4534,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4543,7 +4545,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4554,17 +4556,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4576,7 +4578,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4587,7 +4589,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4598,24 +4600,24 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -4631,7 +4633,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4647,12 +4649,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4664,7 +4666,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4675,7 +4677,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4691,12 +4693,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4708,7 +4710,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4719,7 +4721,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4730,29 +4732,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4763,7 +4765,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4774,17 +4776,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4807,7 +4809,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4825,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4851,7 +4853,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4862,17 +4864,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4895,7 +4897,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4906,17 +4908,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4928,7 +4930,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4939,28 +4941,28 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4972,7 +4974,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4983,28 +4985,28 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5016,7 +5018,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5027,7 +5029,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5050,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5071,28 +5073,28 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5104,7 +5106,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5115,7 +5117,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5126,17 +5128,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5148,7 +5150,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5159,7 +5161,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5170,17 +5172,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5192,7 +5194,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5203,7 +5205,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5219,7 +5221,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5247,7 +5249,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5263,12 +5265,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5291,7 +5293,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5307,7 +5309,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5335,7 +5337,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5346,17 +5348,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5379,7 +5381,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5402,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5423,12 +5425,56 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr"/>
+      <c r="B111" t="n">
+        <v>45</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L110"/>
+  <autoFilter ref="A1:L111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5495,7 +5541,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5595,7 +5641,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C6" t="n">
         <v>89</v>
@@ -5649,68 +5695,68 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABRIO GmbH</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>ABRIO GmbH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>136</v>
+        <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -5724,51 +5770,43 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>93</v>
+        <v>119</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Product Marketing (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>greenhouse</t>
-        </is>
-      </c>
+          <t>Praktikum Brand Management (m/w/d(</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Product Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5778,34 +5816,42 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>smartrecruiters</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+          <t>Category Management Praktikum (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>smartrecruiters</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5815,18 +5861,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -5840,18 +5886,18 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -5865,18 +5911,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -5890,18 +5936,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -5915,18 +5961,18 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -5940,18 +5986,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -5965,25 +6011,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -5994,7 +6040,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C21" t="n">
         <v>83</v>
@@ -6102,7 +6148,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6127,7 +6173,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6152,7 +6198,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6202,7 +6248,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6227,7 +6273,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6285,7 +6331,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6310,7 +6356,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6385,7 +6431,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6485,7 +6531,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6510,7 +6556,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6535,7 +6581,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6560,7 +6606,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -6593,7 +6639,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -6618,7 +6664,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6668,7 +6714,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6701,7 +6747,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6726,7 +6772,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6776,7 +6822,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C51" t="n">
         <v>54</v>
@@ -6801,7 +6847,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6826,7 +6872,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -6976,7 +7022,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -7001,7 +7047,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -7051,7 +7097,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C62" t="n">
         <v>50</v>
@@ -7076,7 +7122,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7101,7 +7147,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7126,7 +7172,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7176,7 +7222,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7201,7 +7247,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -7226,7 +7272,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7276,7 +7322,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7301,7 +7347,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C72" t="n">
         <v>49</v>
@@ -7726,7 +7772,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C89" t="n">
         <v>46</v>
@@ -7776,7 +7822,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C91" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-18 10:45 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -756,12 +756,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -795,7 +795,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -806,31 +806,35 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -841,7 +845,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -857,7 +861,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -876,7 +880,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -887,7 +891,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -903,12 +907,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -922,7 +926,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -933,7 +937,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -944,17 +948,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -968,7 +972,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -979,7 +983,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1004,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1025,36 +1029,34 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1073,36 +1075,34 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>6</v>
-      </c>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1123,7 +1123,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1150,7 +1150,11 @@
       <c r="F15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1169,7 +1173,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1180,17 +1184,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1204,7 +1208,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1215,7 +1219,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1226,27 +1230,23 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>6</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1265,7 +1265,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1286,13 +1286,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1311,7 +1315,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1908,24 +1912,26 @@
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>6</v>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
@@ -1934,7 +1940,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1945,7 +1951,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1967,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1991,7 +1997,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2013,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2018,7 +2024,11 @@
       <c r="F34" t="n">
         <v>6</v>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2037,7 +2047,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2048,17 +2058,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2066,7 +2076,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2087,46 +2097,40 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>6</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2137,40 +2141,40 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2181,7 +2185,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2206,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2225,7 +2229,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2236,17 +2240,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2269,7 +2273,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2280,17 +2284,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2313,7 +2317,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2333,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2346,7 +2350,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2357,7 +2361,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2377,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2390,7 +2394,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2401,7 +2405,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2421,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2434,7 +2438,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2445,51 +2449,55 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="n">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Exclusive Associates</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2632,20 +2640,18 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="n">
+        <v>6</v>
+      </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
@@ -2654,7 +2660,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2665,7 +2671,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2687,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2698,7 +2704,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2709,7 +2715,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2720,12 +2726,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2742,7 +2748,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2753,7 +2759,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -2764,12 +2770,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2786,7 +2792,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2797,40 +2803,40 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2841,28 +2847,28 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2874,7 +2880,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2885,35 +2891,35 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2929,26 +2935,30 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr"/>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
@@ -2958,7 +2968,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2969,33 +2979,31 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>6</v>
-      </c>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
@@ -3015,7 +3023,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3034,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3036,7 +3044,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -3061,31 +3069,33 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>6</v>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3105,7 +3115,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3116,17 +3126,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -3138,7 +3148,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3149,7 +3159,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3160,12 +3170,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3174,11 +3184,7 @@
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3186,7 +3192,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3197,7 +3203,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3208,24 +3214,28 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3241,7 +3251,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3267,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3274,7 +3284,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3285,7 +3295,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3311,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3318,7 +3328,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3329,46 +3339,40 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>6</v>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3379,7 +3383,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3394,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3418,7 +3422,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3429,7 +3433,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3440,29 +3444,35 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>6</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3473,7 +3483,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3484,29 +3494,29 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3517,7 +3527,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3528,12 +3538,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3550,7 +3560,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3561,28 +3571,28 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
       <c r="B69" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
@@ -3594,7 +3604,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3605,7 +3615,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
@@ -3616,25 +3626,21 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3642,7 +3648,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3653,7 +3659,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3664,12 +3670,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3680,7 +3686,7 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3690,7 +3696,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3701,7 +3707,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3723,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3738,7 +3744,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3760,21 +3766,25 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3782,7 +3792,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3793,7 +3803,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3804,17 +3814,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3826,7 +3836,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3837,28 +3847,28 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3870,7 +3880,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3881,7 +3891,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3907,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3906,11 +3916,7 @@
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3918,7 +3924,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3929,7 +3935,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -3940,29 +3946,33 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3973,55 +3983,51 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="n">
+        <v>50</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Richemont</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Internship - High Jewelry Business Development Assistant</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
           <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>Richemont</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr"/>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
@@ -4032,35 +4038,29 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F79" t="n">
-        <v>6</v>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4071,36 +4071,46 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>6</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4111,7 +4121,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4137,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -4140,7 +4150,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4151,7 +4161,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4162,29 +4172,25 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4195,7 +4201,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4222,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4228,7 +4234,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4239,7 +4245,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4250,17 +4256,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4272,7 +4278,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4283,7 +4289,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4294,15 +4300,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
@@ -4312,7 +4322,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4323,7 +4333,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4339,7 +4349,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -4352,7 +4362,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4363,7 +4373,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4374,19 +4384,15 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
@@ -4396,7 +4402,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4407,7 +4413,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4418,17 +4424,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4440,7 +4446,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4451,7 +4457,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4462,17 +4468,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4484,7 +4490,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4495,7 +4501,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4506,24 +4512,24 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4539,7 +4545,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4555,12 +4561,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4572,7 +4578,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4583,7 +4589,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4599,12 +4605,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4616,7 +4622,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4627,7 +4633,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4638,29 +4644,29 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4671,7 +4677,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4682,17 +4688,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4715,7 +4721,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4737,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4759,7 +4765,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4770,17 +4776,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4803,7 +4809,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4814,17 +4820,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4836,7 +4842,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4847,28 +4853,28 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4880,7 +4886,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4891,72 +4897,76 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr"/>
-      <c r="B99" t="n">
-        <v>46</v>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>SUPA - Sport Und Party App</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Business Development Praktikum</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Paris, Paris, France</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4968,7 +4978,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4979,28 +4989,28 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5012,7 +5022,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5023,28 +5033,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5056,7 +5066,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5067,7 +5077,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5078,17 +5088,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5100,7 +5110,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5111,7 +5121,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5122,17 +5132,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5144,7 +5154,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5155,7 +5165,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5186,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5199,7 +5209,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5230,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5243,7 +5253,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5254,17 +5264,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5287,7 +5297,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5298,12 +5308,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5331,12 +5341,100 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr"/>
+      <c r="B109" t="n">
+        <v>45</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr"/>
+      <c r="B110" t="n">
+        <v>45</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L108"/>
+  <autoFilter ref="A1:L110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5403,7 +5501,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5478,7 +5576,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -5561,7 +5659,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -5586,7 +5684,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n">
         <v>87</v>
@@ -5611,7 +5709,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5636,7 +5734,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5661,7 +5759,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5694,7 +5792,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5727,7 +5825,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5752,7 +5850,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -5777,7 +5875,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5802,7 +5900,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -5827,7 +5925,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -5852,7 +5950,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -5902,7 +6000,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C21" t="n">
         <v>83</v>
@@ -6010,7 +6108,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6035,7 +6133,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6060,7 +6158,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6110,7 +6208,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6135,7 +6233,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6193,7 +6291,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6218,7 +6316,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6293,7 +6391,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6393,7 +6491,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6418,7 +6516,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6443,7 +6541,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6468,7 +6566,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -6493,7 +6591,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -6526,7 +6624,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6576,7 +6674,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6609,7 +6707,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6634,7 +6732,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6709,7 +6807,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6734,7 +6832,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -6884,7 +6982,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -6909,7 +7007,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -6984,7 +7082,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7009,7 +7107,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7034,7 +7132,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7055,43 +7153,43 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -7105,7 +7203,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -7116,14 +7214,14 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -7134,7 +7232,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7159,7 +7257,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
@@ -7184,7 +7282,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7634,7 +7732,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C89" t="n">
         <v>46</v>
@@ -7684,7 +7782,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C91" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-19 10:28 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$110</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -756,12 +756,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -795,7 +795,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -806,35 +806,31 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -845,7 +841,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -861,7 +857,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -880,7 +876,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -891,7 +887,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -907,12 +903,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -926,7 +922,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -937,7 +933,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -948,17 +944,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -972,7 +968,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -983,7 +979,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1000,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1029,34 +1025,36 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1075,34 +1073,36 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>6</v>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1123,7 +1123,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1150,11 +1150,7 @@
       <c r="F15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1173,7 +1169,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1180,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1208,7 +1204,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1219,7 +1215,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1230,23 +1226,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>6</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1265,7 +1265,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1286,17 +1286,13 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1315,7 +1311,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1414,27 +1410,21 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HUGO BOSS</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Metzingen, Reutlingen (Kreis)</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1442,7 +1432,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1453,7 +1443,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1464,20 +1454,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>6</v>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
@@ -1497,28 +1489,28 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1532,7 +1524,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1543,7 +1535,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1554,17 +1546,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1578,7 +1570,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1589,32 +1581,32 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
@@ -1624,7 +1616,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1635,7 +1627,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1643,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1681,7 +1673,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1692,21 +1684,21 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
@@ -1716,7 +1708,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1727,33 +1719,31 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>2</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
@@ -1762,7 +1752,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1773,28 +1763,28 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -1806,7 +1796,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1817,7 +1807,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1823,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1850,7 +1840,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1861,7 +1851,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -1882,7 +1872,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1894,7 +1884,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1905,7 +1895,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
@@ -2640,18 +2630,20 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="n">
-        <v>6</v>
-      </c>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
@@ -2660,7 +2652,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2671,7 +2663,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2679,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2704,7 +2696,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2715,7 +2707,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -2726,12 +2718,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2748,7 +2740,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2759,7 +2751,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -2770,12 +2762,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2792,7 +2784,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2803,7 +2795,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
@@ -2814,12 +2806,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2836,7 +2828,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2847,40 +2839,40 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2891,35 +2883,35 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2935,7 +2927,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2948,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2979,30 +2971,26 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
@@ -3012,7 +3000,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3023,7 +3011,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -3664,98 +3652,98 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="n">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Norton Rose Fulbright</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>München, München (Kreis)</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="n">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>SERVICEPLAN Gruppe</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Norton Rose Fulbright</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Altstadt-Lehel, München</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -3766,12 +3754,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3782,7 +3770,7 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3792,7 +3780,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3803,7 +3791,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3814,21 +3802,25 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3836,7 +3828,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3847,7 +3839,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3858,17 +3850,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3880,7 +3872,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3891,28 +3883,28 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3924,7 +3916,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3935,7 +3927,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3943,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3960,11 +3952,7 @@
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3972,7 +3960,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3983,7 +3971,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -3994,29 +3982,33 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4027,7 +4019,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4035,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4060,7 +4052,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4071,7 +4063,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4082,35 +4074,29 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F80" t="n">
-        <v>6</v>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4121,36 +4107,46 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>6</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4161,7 +4157,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4173,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -4190,7 +4186,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4201,7 +4197,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4212,29 +4208,25 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4245,7 +4237,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4258,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4278,7 +4270,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4289,7 +4281,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4300,17 +4292,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4322,7 +4314,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4333,7 +4325,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4344,15 +4336,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
@@ -4362,7 +4358,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4373,7 +4369,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4385,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -4402,7 +4398,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4413,7 +4409,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4424,19 +4420,15 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -4446,7 +4438,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4457,7 +4449,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4468,17 +4460,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4490,7 +4482,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4501,7 +4493,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4512,17 +4504,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4534,7 +4526,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4545,7 +4537,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4556,24 +4548,24 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4589,7 +4581,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4605,12 +4597,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4622,7 +4614,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4633,7 +4625,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4649,12 +4641,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4666,7 +4658,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4677,7 +4669,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4688,29 +4680,29 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4721,7 +4713,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4732,17 +4724,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4765,7 +4757,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4773,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4809,7 +4801,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4820,17 +4812,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4853,7 +4845,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4864,17 +4856,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4886,7 +4878,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4897,120 +4889,120 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="n">
+        <v>49</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Gornhofen, Ravensburg</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B99" s="2" t="n">
+      <c r="B100" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="C99" s="2" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Doctolib</t>
         </is>
       </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="D100" s="2" t="inlineStr">
         <is>
           <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
         </is>
       </c>
-      <c r="E99" s="2" t="inlineStr">
+      <c r="E100" s="2" t="inlineStr">
         <is>
           <t>Paris, Paris, France</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" s="2" t="inlineStr"/>
-      <c r="H99" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I99" s="2" t="inlineStr">
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="J99" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K99" s="2" t="inlineStr"/>
-      <c r="L99" s="2" t="inlineStr">
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr"/>
-      <c r="B100" t="n">
-        <v>48</v>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Konzernzentrale</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5022,7 +5014,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5033,7 +5025,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5046,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5077,28 +5069,28 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5110,7 +5102,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5121,7 +5113,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5132,17 +5124,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5154,7 +5146,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5165,7 +5157,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5445,7 +5437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5501,7 +5493,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5576,7 +5568,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -5659,7 +5651,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -5684,7 +5676,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" t="n">
         <v>87</v>
@@ -5709,7 +5701,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5734,7 +5726,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5759,7 +5751,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5792,7 +5784,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5825,7 +5817,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5850,7 +5842,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -5875,7 +5867,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5900,7 +5892,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -5925,7 +5917,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -5950,7 +5942,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -6000,7 +5992,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C21" t="n">
         <v>83</v>
@@ -6108,7 +6100,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6133,7 +6125,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6158,7 +6150,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6208,7 +6200,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6233,7 +6225,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6291,7 +6283,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6316,7 +6308,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6391,7 +6383,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6491,7 +6483,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6516,7 +6508,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6541,7 +6533,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6566,7 +6558,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -6624,7 +6616,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6674,7 +6666,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6707,7 +6699,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6732,7 +6724,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6807,7 +6799,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6832,7 +6824,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -6982,7 +6974,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -7007,7 +6999,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -7028,93 +7020,93 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>HardyTec Industries UG haftungsbeschränkt</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" t="n">
         <v>51</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C62" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Business Development</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="C63" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -7128,18 +7120,18 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -7153,43 +7145,43 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -7203,161 +7195,161 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Clarios</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C72" t="n">
         <v>49</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Clarios</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C73" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C74" t="n">
         <v>48</v>
@@ -7371,50 +7363,50 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C75" t="n">
         <v>48</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C76" t="n">
         <v>48</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -7428,7 +7420,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -7439,7 +7431,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7453,7 +7445,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7464,7 +7456,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7478,7 +7470,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -7489,7 +7481,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7503,7 +7495,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -7514,7 +7506,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7528,7 +7520,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -7539,7 +7531,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7553,18 +7545,18 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C82" t="n">
         <v>48</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7578,7 +7570,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -7589,7 +7581,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -7603,7 +7595,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -7614,7 +7606,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -7628,7 +7620,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -7639,7 +7631,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -7653,7 +7645,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -7664,7 +7656,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -7678,7 +7670,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -7689,7 +7681,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -7703,7 +7695,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -7714,7 +7706,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -7728,18 +7720,18 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="C89" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -7753,82 +7745,82 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>24</v>
+        <v>98</v>
       </c>
       <c r="C90" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C91" t="n">
         <v>45</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C92" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -7839,7 +7831,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -7853,7 +7845,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -7864,7 +7856,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -7878,18 +7870,18 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C95" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -7903,18 +7895,18 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C96" t="n">
         <v>38</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -7928,7 +7920,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -7939,7 +7931,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -7953,18 +7945,18 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>1</v>
       </c>
       <c r="C98" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -7978,18 +7970,18 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C99" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -8003,18 +7995,18 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C100" t="n">
         <v>28</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -8028,7 +8020,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -8039,7 +8031,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -8053,7 +8045,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -8064,7 +8056,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -8078,7 +8070,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -8089,7 +8081,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -8103,7 +8095,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -8114,7 +8106,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -8128,7 +8120,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -8139,7 +8131,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -8153,7 +8145,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -8164,7 +8156,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -8178,7 +8170,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>AUMOVIO</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -8189,7 +8181,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -8200,8 +8192,33 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" t="n">
+        <v>28</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G107"/>
+  <autoFilter ref="A1:G108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-09-20 10:47 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$110</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -756,12 +756,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -795,7 +795,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -806,31 +806,35 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -841,7 +845,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -857,7 +861,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -876,7 +880,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -887,7 +891,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -903,12 +907,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -922,7 +926,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -933,7 +937,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -944,17 +948,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -968,7 +972,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -979,7 +983,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1004,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1025,36 +1029,34 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1073,36 +1075,34 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>6</v>
-      </c>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1123,7 +1123,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1150,7 +1150,11 @@
       <c r="F15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1169,7 +1173,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1180,17 +1184,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1204,7 +1208,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1215,7 +1219,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1226,27 +1230,23 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>6</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1265,7 +1265,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1286,13 +1286,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1311,7 +1315,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2444,48 +2448,44 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="n">
         <v>62</v>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Exclusive Associates</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -2630,20 +2630,18 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="n">
+        <v>6</v>
+      </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
@@ -2652,7 +2650,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2663,7 +2661,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2677,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2696,7 +2694,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2707,7 +2705,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2718,12 +2716,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2740,7 +2738,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2751,7 +2749,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -2762,12 +2760,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2784,7 +2782,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2795,7 +2793,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2809,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2828,7 +2826,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2839,40 +2837,40 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2883,35 +2881,35 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2927,7 +2925,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2946,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2971,26 +2969,30 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr"/>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
@@ -3000,7 +3002,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3011,7 +3013,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3165,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3180,7 +3182,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3191,7 +3193,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3202,12 +3204,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3216,11 +3218,7 @@
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3228,7 +3226,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3239,7 +3237,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3250,24 +3248,28 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3283,7 +3285,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3299,7 +3301,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3316,7 +3318,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3327,7 +3329,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3345,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3360,7 +3362,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3371,46 +3373,40 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F65" t="n">
-        <v>6</v>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3421,7 +3417,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3428,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3460,7 +3456,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3471,7 +3467,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3482,29 +3478,35 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>6</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3515,7 +3517,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3526,29 +3528,29 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3559,7 +3561,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3570,12 +3572,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3592,7 +3594,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3603,28 +3605,28 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3636,7 +3638,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3647,55 +3649,51 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="n">
+        <v>51</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CHECK24 Vergleichsportal</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development – Shopping</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Mitte, Berlin</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Norton Rose Fulbright</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr"/>
-      <c r="G71" s="2" t="inlineStr"/>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K71" s="2" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3708,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3720,7 +3718,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr"/>
@@ -3732,7 +3730,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3743,103 +3741,103 @@
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Norton Rose Fulbright</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>München, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Norton Rose Fulbright</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Altstadt-Lehel, München</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="n">
-        <v>51</v>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="n">
-        <v>51</v>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>SERVICEPLAN Gruppe</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3850,21 +3848,25 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3883,7 +3885,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3894,21 +3896,25 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3916,7 +3922,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3927,28 +3933,28 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3960,7 +3966,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3971,36 +3977,32 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4008,7 +4010,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4019,7 +4021,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4030,29 +4032,29 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4063,7 +4065,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -4074,29 +4076,33 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4107,7 +4113,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
         </is>
       </c>
     </row>
@@ -4118,35 +4124,29 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F81" t="n">
-        <v>6</v>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4157,26 +4157,30 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr"/>
+          <t>High Jewelry Business Development Assistant Intern</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
@@ -4186,7 +4190,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4197,36 +4201,46 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>6</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4237,7 +4251,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
@@ -4248,29 +4262,25 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4281,7 +4291,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4292,29 +4302,25 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Bult, Hannover</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4325,7 +4331,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4336,17 +4342,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4358,7 +4364,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4369,7 +4375,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4380,15 +4386,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
@@ -4398,7 +4408,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4409,7 +4419,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4435,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -4438,7 +4448,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4449,7 +4459,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4460,19 +4470,15 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -4482,7 +4488,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4493,7 +4499,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4504,17 +4510,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4526,7 +4532,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4537,7 +4543,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4548,17 +4554,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4570,7 +4576,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4581,7 +4587,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4592,24 +4598,24 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -4625,7 +4631,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4641,12 +4647,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4658,7 +4664,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4669,7 +4675,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4685,12 +4691,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4702,7 +4708,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4713,7 +4719,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4724,29 +4730,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4757,7 +4763,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4768,17 +4774,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4801,7 +4807,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4823,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4845,7 +4851,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4856,17 +4862,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4889,7 +4895,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4900,17 +4906,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4922,7 +4928,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4933,55 +4939,51 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr"/>
+      <c r="B100" t="n">
+        <v>49</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Gornhofen, Ravensburg</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>Doctolib</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>Paris, Paris, France</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr"/>
-      <c r="G100" s="2" t="inlineStr"/>
-      <c r="H100" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I100" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="J100" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K100" s="2" t="inlineStr"/>
-      <c r="L100" s="2" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
@@ -4992,17 +4994,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Paris, Paris, France</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5014,7 +5016,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5025,28 +5027,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5058,7 +5060,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5069,7 +5071,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5092,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5113,28 +5115,28 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5146,7 +5148,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5157,7 +5159,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5168,17 +5170,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5190,7 +5192,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5201,7 +5203,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5219,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5245,7 +5247,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5261,12 +5263,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5289,7 +5291,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5305,7 +5307,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5333,7 +5335,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5344,17 +5346,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5377,7 +5379,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5400,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5421,12 +5423,56 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr"/>
+      <c r="B111" t="n">
+        <v>45</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L110"/>
+  <autoFilter ref="A1:L111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5437,7 +5483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5493,7 +5539,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5568,7 +5614,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -5651,7 +5697,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -5676,7 +5722,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" t="n">
         <v>87</v>
@@ -5701,7 +5747,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5726,7 +5772,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5751,7 +5797,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5784,7 +5830,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5817,7 +5863,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5842,7 +5888,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -5867,7 +5913,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5892,7 +5938,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -5917,7 +5963,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -5942,7 +5988,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -5992,7 +6038,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C21" t="n">
         <v>83</v>
@@ -6100,7 +6146,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6125,7 +6171,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6150,7 +6196,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6200,7 +6246,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6225,7 +6271,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6283,7 +6329,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6308,7 +6354,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6383,7 +6429,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6483,7 +6529,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6508,7 +6554,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6533,7 +6579,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6616,7 +6662,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6666,7 +6712,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6699,7 +6745,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6724,7 +6770,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6774,7 +6820,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C51" t="n">
         <v>54</v>
@@ -6799,7 +6845,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6824,7 +6870,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -6974,7 +7020,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -6999,7 +7045,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -7024,7 +7070,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C61" t="n">
         <v>51</v>
@@ -7070,68 +7116,68 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C63" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="B64" t="n">
+        <v>15</v>
+      </c>
+      <c r="C64" t="n">
         <v>50</v>
       </c>
-      <c r="C64" t="n">
-        <v>49</v>
-      </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -7145,18 +7191,18 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -7170,43 +7216,43 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -7220,161 +7266,161 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C72" t="n">
         <v>49</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Clarios</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C73" t="n">
         <v>49</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Clarios</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C74" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C75" t="n">
         <v>48</v>
@@ -7388,50 +7434,50 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C76" t="n">
         <v>48</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C77" t="n">
         <v>48</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7445,7 +7491,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7456,7 +7502,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7470,7 +7516,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -7481,7 +7527,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7495,7 +7541,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -7506,7 +7552,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7520,7 +7566,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -7531,7 +7577,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7545,7 +7591,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -7556,7 +7602,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7570,18 +7616,18 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C83" t="n">
         <v>48</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -7595,7 +7641,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -7606,7 +7652,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -7620,7 +7666,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -7631,7 +7677,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -7645,7 +7691,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -7656,7 +7702,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -7670,7 +7716,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -7681,7 +7727,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -7695,7 +7741,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -7706,7 +7752,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -7720,7 +7766,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -7731,7 +7777,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -7745,18 +7791,18 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
       <c r="C90" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -7770,82 +7816,82 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="C91" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C92" t="n">
         <v>45</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C93" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -7856,7 +7902,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -7870,7 +7916,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -7881,7 +7927,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -7895,18 +7941,18 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C96" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -7920,18 +7966,18 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C97" t="n">
         <v>38</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -7945,7 +7991,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -7956,7 +8002,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -7970,18 +8016,18 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>1</v>
       </c>
       <c r="C99" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -7995,18 +8041,18 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C100" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -8020,18 +8066,18 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C101" t="n">
         <v>28</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -8045,7 +8091,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -8056,7 +8102,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -8070,7 +8116,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -8081,7 +8127,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -8095,7 +8141,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -8106,7 +8152,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -8120,7 +8166,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -8131,7 +8177,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -8145,7 +8191,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -8156,7 +8202,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -8170,7 +8216,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -8181,7 +8227,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -8195,7 +8241,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>AUMOVIO</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -8206,7 +8252,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -8217,8 +8263,33 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>1</v>
+      </c>
+      <c r="C109" t="n">
+        <v>28</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G108"/>
+  <autoFilter ref="A1:G109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-09-21 12:10 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -706,25 +706,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -745,7 +745,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -756,17 +756,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -774,7 +774,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -795,7 +795,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -806,12 +806,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -845,7 +845,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -856,31 +856,35 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -891,7 +895,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1787,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1800,7 +1804,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1811,31 +1815,33 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>6</v>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
@@ -1844,7 +1850,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1855,31 +1861,33 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>6</v>
+      </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
@@ -1888,7 +1896,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1899,7 +1907,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1923,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1926,7 +1934,11 @@
       <c r="F32" t="n">
         <v>6</v>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1945,7 +1957,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1956,23 +1968,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>6</v>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1991,38 +2007,32 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>6</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2041,46 +2051,40 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>6</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2091,40 +2095,40 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2135,7 +2139,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2160,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2179,7 +2183,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2190,17 +2194,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2223,7 +2227,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2234,17 +2238,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2267,7 +2271,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2283,7 +2287,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2300,7 +2304,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2311,7 +2315,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2331,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2344,7 +2348,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2355,7 +2359,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2375,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2388,7 +2392,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2399,7 +2403,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2419,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2432,7 +2436,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2443,7 +2447,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2454,17 +2458,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2476,7 +2480,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2487,7 +2491,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2512,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2531,28 +2535,28 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2575,31 +2579,29 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>6</v>
+      </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
@@ -2608,7 +2610,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2619,7 +2621,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -2630,18 +2632,20 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="n">
-        <v>6</v>
-      </c>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
@@ -2650,7 +2654,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2661,7 +2665,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -2672,12 +2676,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2705,7 +2709,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -2716,12 +2720,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2738,7 +2742,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2749,7 +2753,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
@@ -2760,12 +2764,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2782,7 +2786,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2793,7 +2797,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2813,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2826,7 +2830,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2837,40 +2841,40 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2881,35 +2885,35 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2925,7 +2929,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2950,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2969,31 +2973,33 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>6</v>
+      </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
@@ -3013,7 +3019,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3030,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3034,7 +3040,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -3059,33 +3065,31 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3105,7 +3109,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3116,17 +3120,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -3138,7 +3142,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3149,7 +3153,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3160,24 +3164,24 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3193,7 +3197,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3204,29 +3208,29 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3237,7 +3241,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
@@ -3248,33 +3252,29 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3285,40 +3285,46 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>6</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3329,40 +3335,46 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>6</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3373,40 +3385,40 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3417,7 +3429,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3428,27 +3440,21 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>6</v>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3456,7 +3462,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3467,7 +3473,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3478,27 +3484,21 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F67" t="n">
-        <v>6</v>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3517,40 +3517,40 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3561,72 +3561,76 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="n">
-        <v>52</v>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Wonder Natural GmbH</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>NRF</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>München, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3638,7 +3642,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3649,7 +3653,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -3660,17 +3664,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3682,7 +3686,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3693,151 +3697,147 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="n">
         <v>51</v>
       </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>NRF</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>München, München (Kreis)</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="n">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="n">
         <v>51</v>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Norton Rose Fulbright</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SERVICEPLAN Gruppe</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>München, München (Kreis)</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K73" s="2" t="inlineStr"/>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="n">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="n">
         <v>51</v>
       </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Norton Rose Fulbright</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>WirWinzer</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>Altstadt-Lehel, München</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3848,25 +3848,21 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3874,7 +3870,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3885,36 +3881,32 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3922,7 +3914,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3933,32 +3925,36 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3966,7 +3962,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3977,40 +3973,40 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4021,7 +4017,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4032,29 +4028,29 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4065,7 +4061,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
@@ -4076,20 +4072,22 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr"/>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>6</v>
+      </c>
       <c r="G80" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -4102,7 +4100,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4113,30 +4111,26 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
@@ -4146,7 +4140,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4157,30 +4151,26 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
@@ -4190,7 +4180,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4201,38 +4191,32 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F83" t="n">
-        <v>6</v>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Hannover, Region Hannover (Kreis)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4240,7 +4224,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4251,7 +4235,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4262,25 +4246,29 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4291,7 +4279,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4302,12 +4290,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -4315,12 +4303,12 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4331,7 +4319,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4342,19 +4330,15 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
@@ -4364,7 +4348,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4375,7 +4359,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4386,17 +4370,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4408,7 +4392,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4419,7 +4403,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4430,15 +4414,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr"/>
+          <t>Praktikum Category Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Münster, Nordrhein-Westfalen</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -4448,7 +4436,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4459,7 +4447,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4470,15 +4458,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -4488,7 +4480,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4499,7 +4491,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4510,17 +4502,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4532,7 +4524,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4543,7 +4535,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4554,29 +4546,29 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4587,7 +4579,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4598,29 +4590,29 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4631,7 +4623,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4639,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4664,7 +4656,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4686,29 +4678,29 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4719,7 +4711,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4730,29 +4722,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4763,7 +4755,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4774,17 +4766,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4807,7 +4799,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4818,17 +4810,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4851,7 +4843,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4862,17 +4854,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4884,7 +4876,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4895,28 +4887,28 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr"/>
       <c r="B99" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Paris, Paris, France</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4928,7 +4920,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4939,28 +4931,28 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4972,7 +4964,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4983,28 +4975,28 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Paris, Paris, France</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5016,7 +5008,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5027,28 +5019,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5060,7 +5052,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5071,28 +5063,28 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5104,7 +5096,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5115,28 +5107,28 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5159,7 +5151,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5170,17 +5162,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5192,7 +5184,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5203,7 +5195,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5216,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5247,7 +5239,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5260,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5291,7 +5283,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5302,17 +5294,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5335,7 +5327,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5346,12 +5338,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5379,100 +5371,12 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr"/>
-      <c r="B110" t="n">
-        <v>45</v>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J110" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr"/>
-      <c r="B111" t="n">
-        <v>45</v>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L111"/>
+  <autoFilter ref="A1:L109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5539,7 +5443,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5589,7 +5493,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C4" t="n">
         <v>91</v>
@@ -5614,7 +5518,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -5697,7 +5601,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -5722,7 +5626,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" t="n">
         <v>87</v>
@@ -5747,7 +5651,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5772,7 +5676,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5797,7 +5701,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5830,7 +5734,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5863,7 +5767,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5888,7 +5792,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -5913,7 +5817,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5938,7 +5842,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -5963,7 +5867,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -5988,7 +5892,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -6038,7 +5942,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C21" t="n">
         <v>83</v>
@@ -6146,7 +6050,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6171,7 +6075,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6196,7 +6100,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6246,7 +6150,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6271,7 +6175,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6329,7 +6233,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6354,7 +6258,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6429,7 +6333,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6529,7 +6433,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6554,7 +6458,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6579,7 +6483,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6662,7 +6566,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6712,7 +6616,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6745,7 +6649,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6770,7 +6674,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6820,7 +6724,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C51" t="n">
         <v>54</v>
@@ -6845,7 +6749,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6870,7 +6774,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -7020,7 +6924,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -7045,7 +6949,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -7070,7 +6974,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C61" t="n">
         <v>51</v>
@@ -7091,32 +6995,32 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>HardyTec Industries UG haftungsbeschränkt</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C62" t="n">
         <v>51</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -7127,14 +7031,14 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Marketing &amp; Business Development</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7074,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7195,7 +7099,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -7220,7 +7124,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7245,7 +7149,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -7270,7 +7174,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7320,7 +7224,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7345,7 +7249,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C72" t="n">
         <v>49</v>
@@ -7370,7 +7274,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C73" t="n">
         <v>49</v>
@@ -7820,7 +7724,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C91" t="n">
         <v>46</v>
@@ -7870,7 +7774,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C93" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-22 11:09 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$107</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,11 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D8F3DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,12 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1458,21 +1452,21 @@
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1486,7 +1480,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1497,7 +1491,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1508,17 +1502,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1532,7 +1526,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1543,32 +1537,32 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
@@ -1578,7 +1572,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1589,7 +1583,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1599,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1635,7 +1629,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1646,21 +1640,21 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
@@ -1670,7 +1664,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1681,33 +1675,31 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>2</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
@@ -1716,7 +1708,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1727,28 +1719,28 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1760,7 +1752,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1771,31 +1763,33 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>6</v>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
@@ -1804,7 +1798,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1815,7 +1809,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1825,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1861,7 +1855,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1871,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1888,7 +1882,11 @@
       <c r="F31" t="n">
         <v>6</v>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1907,7 +1905,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1916,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1936,7 +1934,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1957,7 +1955,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1968,27 +1966,23 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>6</v>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2007,7 +2001,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2102,28 +2096,34 @@
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2139,7 +2139,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2183,7 +2183,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2194,17 +2194,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2227,7 +2227,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2238,17 +2238,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2271,7 +2271,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2315,7 +2315,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2359,7 +2359,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2403,7 +2403,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2447,7 +2447,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2458,17 +2458,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2491,7 +2491,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2535,28 +2535,28 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2579,7 +2579,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3197,7 +3197,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3241,40 +3241,46 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>6</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3285,7 +3291,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3296,35 +3302,29 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>6</v>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>MILAN</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3335,7 +3335,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3346,27 +3346,21 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>6</v>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3374,7 +3368,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3385,7 +3379,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3396,29 +3390,29 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3429,28 +3423,28 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -3462,7 +3456,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3473,28 +3467,28 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3506,7 +3500,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3517,7 +3511,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3528,17 +3522,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3550,7 +3544,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3561,55 +3555,51 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="n">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="n">
         <v>51</v>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>NRF</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Norton Rose Fulbright</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="J69" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K69" s="2" t="inlineStr"/>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Altstadt-Lehel, München</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -3620,12 +3610,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3634,7 +3624,11 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3642,7 +3636,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3653,7 +3647,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3664,21 +3658,25 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3686,7 +3684,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3697,7 +3695,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3708,25 +3706,21 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3745,7 +3739,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3756,25 +3750,21 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3782,7 +3772,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3793,28 +3783,28 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3826,7 +3816,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3837,32 +3827,36 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3870,7 +3864,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3881,7 +3875,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
         </is>
       </c>
     </row>
@@ -3892,29 +3886,29 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3925,7 +3919,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -3936,33 +3930,29 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3973,7 +3963,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
@@ -3984,29 +3974,35 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>6</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4017,30 +4013,26 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
@@ -4050,7 +4042,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4061,46 +4053,36 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F80" t="n">
-        <v>6</v>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4111,7 +4093,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4122,25 +4104,29 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Hannover, Region Hannover (Kreis)</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4151,7 +4137,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4162,25 +4148,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4191,7 +4181,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4202,19 +4192,15 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
@@ -4224,7 +4210,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4235,7 +4221,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4246,19 +4232,15 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Unterbilk, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Skincare Merchandising Intern</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
@@ -4268,7 +4250,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4279,7 +4261,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4290,15 +4272,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr"/>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Berlin, Berlin, Germany</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
@@ -4308,7 +4294,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4319,7 +4305,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4330,15 +4316,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr"/>
+          <t>Praktikum Category Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Münster, Nordrhein-Westfalen</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
@@ -4348,7 +4338,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4359,7 +4349,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4370,17 +4360,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4392,7 +4382,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4403,7 +4393,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4414,17 +4404,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4436,7 +4426,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4447,7 +4437,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4458,29 +4448,29 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4491,7 +4481,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4502,29 +4492,29 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4535,7 +4525,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4541,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4568,7 +4558,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4590,29 +4580,29 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4623,7 +4613,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4634,29 +4624,29 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4667,7 +4657,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4678,17 +4668,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4711,7 +4701,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4722,17 +4712,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4755,7 +4745,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4766,17 +4756,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4788,7 +4778,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4799,28 +4789,28 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr"/>
       <c r="B97" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Paris, Paris, France</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4832,7 +4822,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4843,28 +4833,28 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4876,7 +4866,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4887,28 +4877,28 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr"/>
       <c r="B99" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Paris, Paris, France</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4920,7 +4910,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4931,28 +4921,28 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4964,7 +4954,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4975,28 +4965,28 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5008,7 +4998,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5019,28 +5009,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5063,7 +5053,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5074,17 +5064,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5096,7 +5086,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5107,7 +5097,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5118,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5151,7 +5141,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5172,7 +5162,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5195,7 +5185,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5206,17 +5196,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5239,7 +5229,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5250,12 +5240,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5283,100 +5273,12 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr"/>
-      <c r="B108" t="n">
-        <v>45</v>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr"/>
-      <c r="B109" t="n">
-        <v>45</v>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L109"/>
+  <autoFilter ref="A1:L107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5400,37 +5302,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Unternehmen</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Treffer</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Bester Score</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Beispielrolle</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Wird überwacht</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Zuerst gesehen</t>
         </is>
@@ -5443,7 +5345,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5493,7 +5395,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C4" t="n">
         <v>91</v>
@@ -5518,7 +5420,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -5601,7 +5503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -5626,7 +5528,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
         <v>87</v>
@@ -5651,7 +5553,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5676,7 +5578,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5701,7 +5603,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5734,7 +5636,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5767,7 +5669,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5792,7 +5694,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -5817,7 +5719,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5842,7 +5744,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -5867,7 +5769,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -5892,7 +5794,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -5942,7 +5844,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C21" t="n">
         <v>83</v>
@@ -6050,7 +5952,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6075,7 +5977,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C26" t="n">
         <v>78</v>
@@ -6100,7 +6002,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6150,7 +6052,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -6175,7 +6077,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6233,7 +6135,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6258,7 +6160,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -6333,7 +6235,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -6433,7 +6335,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -6458,7 +6360,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -6483,7 +6385,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6566,7 +6468,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6616,7 +6518,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -6649,7 +6551,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -6674,7 +6576,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -6724,7 +6626,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C51" t="n">
         <v>54</v>
@@ -6749,7 +6651,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -6774,7 +6676,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -6924,7 +6826,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C59" t="n">
         <v>51</v>
@@ -6949,7 +6851,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C60" t="n">
         <v>51</v>
@@ -6974,7 +6876,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C61" t="n">
         <v>51</v>
@@ -6999,7 +6901,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C62" t="n">
         <v>51</v>
@@ -7074,7 +6976,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7099,7 +7001,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -7124,7 +7026,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7149,7 +7051,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -7174,7 +7076,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7195,32 +7097,32 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -7231,14 +7133,14 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -7249,7 +7151,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C72" t="n">
         <v>49</v>
@@ -7274,7 +7176,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C73" t="n">
         <v>49</v>
@@ -7724,7 +7626,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C91" t="n">
         <v>46</v>
@@ -7774,7 +7676,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C93" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-28 13:05 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -518,16 +518,16 @@
     <row r="2">
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="n">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -536,9 +536,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -546,7 +550,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -557,7 +561,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -568,21 +572,21 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Düsseldorf</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Landstraße, Wien</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
@@ -592,7 +596,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -603,7 +607,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -614,7 +618,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Österreich</t>
+          <t>Peek &amp; Cloppenburg Düsseldorf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -624,7 +628,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Innere Stadt, Wien</t>
+          <t>Landstraße, Wien</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -638,7 +642,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -649,7 +653,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
+          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -670,7 +674,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Innere Stadt, Wien</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -684,7 +688,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -695,32 +699,32 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
+          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ABRIO GmbH</t>
+          <t>Peek &amp; Cloppenburg Österreich</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bockenheim, Frankfurt am Main</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
@@ -730,7 +734,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -741,28 +745,28 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>ABRIO GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Bockenheim, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -776,7 +780,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -787,7 +791,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -798,17 +802,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -833,107 +837,103 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="n">
+        <v>84</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PRAKTIKUM // Business Development</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Mitte, Berlin</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B10" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>L’ORÉAL</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>PRAKTIKUM (M/W/D) Product Marketing &amp; Brand Communication bei YSL (Luxe Division) - Start Mai für 6 Monate</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5899340175?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="n">
-        <v>84</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Nespresso Deutschland GmbH</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -944,17 +944,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -983,7 +983,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1318,54 +1318,50 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="n">
         <v>78</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>L’ORÉAL</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab Februar/März/April für 6 Monate</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="F19" t="n">
         <v>6</v>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5897975480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -2572,94 +2568,92 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="n">
+        <v>59</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Coty</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="n">
+        <v>6</v>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
+      <c r="B47" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="n">
-        <v>59</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2669,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2692,7 +2686,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2703,7 +2697,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
@@ -2714,12 +2708,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2736,7 +2730,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2747,40 +2741,40 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502880?se=EIPLzwe48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0668B6260348B06F79C79FBD16FB7D4160F27AC4</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2791,40 +2785,40 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5895502880?se=EIPLzwe48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0668B6260348B06F79C79FBD16FB7D4160F27AC4</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2835,7 +2829,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -2846,12 +2840,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,7 +2862,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2879,7 +2873,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2894,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2923,26 +2917,30 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr"/>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
@@ -2952,7 +2950,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2963,7 +2961,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4522,132 +4520,120 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="n">
+      <c r="A90" t="inlineStr"/>
+      <c r="B90" t="n">
         <v>49</v>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>Coty</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D90" t="inlineStr">
         <is>
           <t>Internship / Trade Marketing Europe</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr"/>
-      <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="2" t="inlineStr"/>
-      <c r="H90" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I90" s="2" t="inlineStr">
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J90" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K90" s="2" t="inlineStr"/>
-      <c r="L90" s="2" t="inlineStr">
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
         <is>
           <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="n">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="n">
         <v>49</v>
       </c>
-      <c r="C91" s="2" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Coty</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
         </is>
       </c>
-      <c r="E91" s="2" t="inlineStr"/>
-      <c r="F91" s="2" t="inlineStr"/>
-      <c r="G91" s="2" t="inlineStr"/>
-      <c r="H91" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I91" s="2" t="inlineStr">
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J91" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K91" s="2" t="inlineStr"/>
-      <c r="L91" s="2" t="inlineStr">
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
         <is>
           <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="n">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="n">
         <v>49</v>
       </c>
-      <c r="C92" s="2" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>Coty</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>Internship / Skincare Merchandising</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr"/>
-      <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="2" t="inlineStr"/>
-      <c r="H92" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I92" s="2" t="inlineStr">
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K92" s="2" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr">
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
         <is>
           <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
         </is>
@@ -5094,48 +5080,44 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="n">
+      <c r="A103" t="inlineStr"/>
+      <c r="B103" t="n">
         <v>49</v>
       </c>
-      <c r="C103" s="2" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>Nestle Deutschland</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="D103" t="inlineStr">
         <is>
           <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
         </is>
       </c>
-      <c r="E103" s="2" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>Brussels, BE</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr"/>
-      <c r="G103" s="2" t="inlineStr"/>
-      <c r="H103" s="2" t="inlineStr">
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I103" s="2" t="inlineStr">
+      <c r="I103" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J103" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K103" s="2" t="inlineStr"/>
-      <c r="L103" s="2" t="inlineStr">
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr">
         <is>
           <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
         </is>
@@ -5913,7 +5895,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5938,7 +5920,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -5963,7 +5945,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" t="n">
         <v>107</v>
@@ -5988,7 +5970,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" t="n">
         <v>91</v>
@@ -6013,7 +5995,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C6" t="n">
         <v>89</v>
@@ -6071,7 +6053,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -6121,7 +6103,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C10" t="n">
         <v>89</v>
@@ -6146,7 +6128,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" t="n">
         <v>89</v>
@@ -6179,7 +6161,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12" t="n">
         <v>87</v>
@@ -6204,7 +6186,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6229,7 +6211,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6254,7 +6236,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6287,7 +6269,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6320,7 +6302,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6345,7 +6327,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -6370,7 +6352,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -6395,7 +6377,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
@@ -6420,7 +6402,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C21" t="n">
         <v>84</v>
@@ -6495,7 +6477,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C24" t="n">
         <v>83</v>
@@ -6603,7 +6585,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C28" t="n">
         <v>78</v>
@@ -6628,7 +6610,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C29" t="n">
         <v>78</v>
@@ -6653,7 +6635,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C30" t="n">
         <v>77</v>
@@ -6678,7 +6660,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C31" t="n">
         <v>77</v>
@@ -6703,7 +6685,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C32" t="n">
         <v>74</v>
@@ -6753,7 +6735,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C34" t="n">
         <v>73</v>
@@ -6778,7 +6760,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C35" t="n">
         <v>73</v>
@@ -6836,7 +6818,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C37" t="n">
         <v>72</v>
@@ -6861,7 +6843,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C38" t="n">
         <v>72</v>
@@ -6936,7 +6918,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C41" t="n">
         <v>68</v>
@@ -7011,7 +6993,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C44" t="n">
         <v>65</v>
@@ -7036,7 +7018,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C45" t="n">
         <v>64</v>
@@ -7061,7 +7043,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C46" t="n">
         <v>62</v>
@@ -7086,7 +7068,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C47" t="n">
         <v>62</v>
@@ -7144,7 +7126,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C49" t="n">
         <v>60</v>
@@ -7177,7 +7159,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C50" t="n">
         <v>59</v>
@@ -7198,32 +7180,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Nahrungs- &amp; Genussmittel Karriere</t>
+          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C51" t="n">
         <v>59</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
+          <t>Nahrungs- &amp; Genussmittel Karriere</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -7234,14 +7216,14 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7234,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C53" t="n">
         <v>59</v>
@@ -7277,7 +7259,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C54" t="n">
         <v>57</v>
@@ -7310,7 +7292,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C55" t="n">
         <v>56</v>
@@ -7335,7 +7317,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C56" t="n">
         <v>56</v>
@@ -7360,7 +7342,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C57" t="n">
         <v>55</v>
@@ -7410,7 +7392,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C59" t="n">
         <v>54</v>
@@ -7435,7 +7417,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C60" t="n">
         <v>53</v>
@@ -7460,7 +7442,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C61" t="n">
         <v>53</v>
@@ -7560,7 +7542,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C65" t="n">
         <v>51</v>
@@ -7585,7 +7567,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C66" t="n">
         <v>51</v>
@@ -7660,7 +7642,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -7685,7 +7667,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
@@ -7710,7 +7692,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7735,7 +7717,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C72" t="n">
         <v>49</v>
@@ -7760,7 +7742,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C73" t="n">
         <v>49</v>
@@ -7785,7 +7767,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C74" t="n">
         <v>49</v>
@@ -7806,32 +7788,32 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C75" t="n">
         <v>49</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -7842,14 +7824,14 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -7885,7 +7867,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C78" t="n">
         <v>49</v>
@@ -8335,7 +8317,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C96" t="n">
         <v>46</v>
@@ -8385,7 +8367,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C98" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-02 12:04 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$120</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1130,48 +1130,52 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="n">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Nestle Deutschland</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant (m/w/d) Retail &amp; Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Duesseldorf, DE</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Duesseldorf-Praktikant-%28mwd%29-Retail-&amp;-Trade-Marketing/1443408333/</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1186,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1206,7 +1210,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1217,7 +1221,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1242,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1263,28 +1267,28 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1309,14 +1313,14 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1325,7 +1329,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1336,11 +1340,7 @@
       <c r="F19" t="n">
         <v>6</v>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1359,7 +1359,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1370,23 +1370,27 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>6</v>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1394,7 +1398,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1405,7 +1409,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1416,27 +1420,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab Februar/März/April für 6 Monate</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>6</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2027-04-01</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1455,7 +1455,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5897975480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1466,17 +1466,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing (m/w/d)</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab Februar/März/April für 6 Monate</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1484,17 +1484,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-04-01</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1505,28 +1505,28 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
+          <t>https://www.adzuna.de/details/5897975480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
+          <t>Praktikum Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1555,7 +1555,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1605,32 +1605,38 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1638,7 +1644,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1649,7 +1655,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1660,17 +1666,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -1693,7 +1699,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1715,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1726,7 +1732,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1737,7 +1743,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1748,17 +1754,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1781,23 +1787,23 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1805,9 +1811,7 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>6</v>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
@@ -1816,7 +1820,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1827,7 +1831,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
@@ -2104,24 +2108,26 @@
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>6</v>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
@@ -2130,7 +2136,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2141,7 +2147,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2163,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2187,7 +2193,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2209,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2214,7 +2220,11 @@
       <c r="F38" t="n">
         <v>6</v>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2233,7 +2243,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2244,27 +2254,23 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>6</v>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2283,7 +2289,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2472,48 +2478,44 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="n">
         <v>64</v>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Mars</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Internship in Trade Marketing Royal Canin</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
         <is>
           <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
@@ -2698,31 +2700,25 @@
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Aumovio</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development und Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Regensburg, Regensburg (Kreis)</t>
-        </is>
-      </c>
-      <c r="F49" t="n">
-        <v>6</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>2027-03-01</t>
-        </is>
-      </c>
+          <t>Wedding, Berlin</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2730,7 +2726,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2741,30 +2737,38 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5894317981?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Aumovio</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr"/>
+          <t>Praktikum - Business Development und Marketing</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Regensburg, Regensburg (Kreis)</t>
+        </is>
+      </c>
       <c r="F50" t="n">
         <v>6</v>
       </c>
-      <c r="G50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2772,7 +2776,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2783,7 +2787,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5894317981?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2794,20 +2798,18 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="n">
+        <v>6</v>
+      </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
@@ -2816,7 +2818,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2827,7 +2829,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -2838,12 +2840,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2860,7 +2862,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2871,40 +2873,40 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2915,28 +2917,28 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2948,7 +2950,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2959,35 +2961,35 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3003,7 +3005,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -3014,17 +3016,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3036,7 +3038,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3047,33 +3049,31 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F57" t="n">
-        <v>6</v>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
@@ -3093,55 +3093,51 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Richemont</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>SINGAPORE</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="n">
+        <v>56</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Upsters Energy GmbH</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3148,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3162,7 +3158,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -3187,40 +3183,40 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>SINGAPORE</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3231,31 +3227,33 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>6</v>
+      </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
@@ -3264,7 +3262,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3275,7 +3273,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3286,24 +3284,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3319,7 +3317,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3330,29 +3328,29 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3363,35 +3361,35 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3407,40 +3405,40 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3451,76 +3449,72 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>AUTO1 Group</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (d/m/w)</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="n">
+        <v>52</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Richemont</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>MILAN</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3532,7 +3526,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3543,51 +3537,55 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
-      <c r="B68" t="n">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>NRF</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>AUTO1 Group</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development (d/m/w)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3598,17 +3596,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
@@ -3620,7 +3618,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3631,7 +3629,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3640,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3664,7 +3662,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3675,7 +3673,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3684,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3696,7 +3694,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3708,7 +3706,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3719,7 +3717,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3738,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -3752,7 +3750,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3763,7 +3761,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3782,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3796,7 +3794,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3807,7 +3805,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -3828,7 +3826,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pempelfort, Düsseldorf</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3851,7 +3849,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
+          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3870,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Neustadt, Hamburg</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3895,7 +3893,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
+          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
         </is>
       </c>
     </row>
@@ -3906,25 +3904,21 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Pempelfort, Düsseldorf</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3932,7 +3926,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3943,7 +3937,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
         </is>
       </c>
     </row>
@@ -3954,17 +3948,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Neustadt, Hamburg</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3976,7 +3970,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3987,7 +3981,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
         </is>
       </c>
     </row>
@@ -3998,21 +3992,25 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4020,7 +4018,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4031,28 +4029,28 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4064,7 +4062,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4075,36 +4073,32 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4112,7 +4106,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4123,7 +4117,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4134,29 +4128,29 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4167,7 +4161,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4177,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4200,7 +4194,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4211,26 +4205,30 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr"/>
+          <t>High Jewelry Business Development Assistant Intern</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
@@ -4240,7 +4238,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4251,7 +4249,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
@@ -4262,29 +4260,25 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4295,7 +4289,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4306,17 +4300,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4328,7 +4322,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4339,7 +4333,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4350,15 +4344,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
@@ -4368,7 +4366,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4379,7 +4377,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4393,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -4408,7 +4406,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4419,7 +4417,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4433,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Internship / Trade Marketing Europe</t>
+          <t>Operational Trade Marketing Intern</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -4448,7 +4446,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4459,7 +4457,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4473,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
+          <t>Skincare Merchandising Intern</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -4488,7 +4486,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4499,7 +4497,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4513,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Internship / Skincare Merchandising</t>
+          <t>Internship / Trade Marketing Europe</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -4539,7 +4537,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
         </is>
       </c>
     </row>
@@ -4550,19 +4548,15 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Münster, Nordrhein-Westfalen</t>
-        </is>
-      </c>
+          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
@@ -4572,7 +4566,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4583,7 +4577,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
         </is>
       </c>
     </row>
@@ -4594,19 +4588,15 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Internship / Skincare Merchandising</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
@@ -4616,7 +4606,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4627,7 +4617,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4638,17 +4628,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4660,7 +4650,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4671,7 +4661,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4682,29 +4672,29 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4715,7 +4705,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4726,29 +4716,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4759,7 +4749,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4770,29 +4760,29 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4803,7 +4793,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4814,29 +4804,29 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4847,7 +4837,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4858,29 +4848,29 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4891,7 +4881,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4902,29 +4892,29 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nestlé Baby</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4935,7 +4925,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
+          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4941,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nutrition</t>
+          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4968,7 +4958,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4979,7 +4969,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
         </is>
       </c>
     </row>
@@ -4995,7 +4985,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
+          <t>Brand Manager Intern - Nestlé Baby</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5012,7 +5002,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5023,55 +5013,51 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="n">
+      <c r="A102" t="inlineStr"/>
+      <c r="B102" t="n">
         <v>49</v>
       </c>
-      <c r="C102" s="2" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>Nestle Deutschland</t>
         </is>
       </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Brand Manager Intern - Nutrition</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
         <is>
           <t>Brussels, BE</t>
         </is>
       </c>
-      <c r="F102" s="2" t="inlineStr"/>
-      <c r="G102" s="2" t="inlineStr"/>
-      <c r="H102" s="2" t="inlineStr">
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I102" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="J102" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K102" s="2" t="inlineStr"/>
-      <c r="L102" s="2" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
         </is>
       </c>
     </row>
@@ -5082,29 +5068,29 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5115,51 +5101,55 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr"/>
-      <c r="B104" t="n">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Nestle Deutschland</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Brussels, BE</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
         </is>
       </c>
     </row>
@@ -5170,17 +5160,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5203,7 +5193,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -5214,17 +5204,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5236,7 +5226,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5247,7 +5237,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -5258,17 +5248,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Rankweil, Feldkirch</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5280,7 +5270,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5291,7 +5281,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5896357793?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA0A29D7B49D4A241A4DCD6CB490D5AA41F3E792</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5302,17 +5292,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Reckitt</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (all genders)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Heidelberg, Baden-Württemberg</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5324,7 +5314,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5335,28 +5325,28 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr"/>
       <c r="B109" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Paris, Paris, France</t>
+          <t>Rankweil, Feldkirch</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5368,7 +5358,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -5379,28 +5369,28 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
+          <t>https://www.adzuna.at/land/ad/5896357793?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA0A29D7B49D4A241A4DCD6CB490D5AA41F3E792</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr"/>
       <c r="B110" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Brand Marketing (all genders)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Heidelberg, Baden-Württemberg</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5412,7 +5402,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -5423,28 +5413,28 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr"/>
       <c r="B111" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Paris, Paris, France</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -5456,7 +5446,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5467,28 +5457,28 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr"/>
       <c r="B112" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5500,7 +5490,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -5511,28 +5501,28 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr"/>
       <c r="B113" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5555,7 +5545,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5566,17 +5556,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5588,7 +5578,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -5599,7 +5589,7 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5620,7 +5610,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5643,7 +5633,7 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5664,7 +5654,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5687,7 +5677,7 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5698,17 +5688,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5731,7 +5721,7 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5742,12 +5732,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5775,12 +5765,100 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="n">
+        <v>45</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr"/>
+      <c r="B120" t="n">
+        <v>45</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L118"/>
+  <autoFilter ref="A1:L120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5847,7 +5925,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -5872,7 +5950,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -5897,7 +5975,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" t="n">
         <v>107</v>
@@ -5972,7 +6050,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="C7" t="n">
         <v>89</v>
@@ -6030,7 +6108,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C9" t="n">
         <v>89</v>
@@ -6051,32 +6129,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VEYNOU GmbH</t>
+          <t>Peek &amp; Cloppenburg Österreich</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C10" t="n">
         <v>89</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
+          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Österreich</t>
+          <t>VEYNOU GmbH</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -6087,14 +6165,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6183,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" t="n">
         <v>89</v>
@@ -6138,7 +6216,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" t="n">
         <v>87</v>
@@ -6171,7 +6249,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" t="n">
         <v>87</v>
@@ -6196,7 +6274,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6221,7 +6299,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6246,7 +6324,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6279,7 +6357,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -6312,7 +6390,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -6337,7 +6415,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
@@ -6362,7 +6440,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C21" t="n">
         <v>84</v>
@@ -6387,7 +6465,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C22" t="n">
         <v>84</v>
@@ -6412,7 +6490,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
         <v>84</v>
@@ -6487,7 +6565,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C26" t="n">
         <v>83</v>
@@ -6595,7 +6673,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C30" t="n">
         <v>78</v>
@@ -6620,7 +6698,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C31" t="n">
         <v>78</v>
@@ -6645,7 +6723,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C32" t="n">
         <v>77</v>
@@ -6670,7 +6748,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C33" t="n">
         <v>77</v>
@@ -6770,7 +6848,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C37" t="n">
         <v>73</v>
@@ -6795,7 +6873,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C38" t="n">
         <v>73</v>
@@ -6878,7 +6956,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C41" t="n">
         <v>72</v>
@@ -6953,7 +7031,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C44" t="n">
         <v>68</v>
@@ -7028,7 +7106,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C47" t="n">
         <v>65</v>
@@ -7053,7 +7131,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C48" t="n">
         <v>64</v>
@@ -7078,7 +7156,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C49" t="n">
         <v>64</v>
@@ -7103,7 +7181,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C50" t="n">
         <v>62</v>
@@ -7128,7 +7206,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C51" t="n">
         <v>62</v>
@@ -7153,7 +7231,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C52" t="n">
         <v>60</v>
@@ -7211,7 +7289,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C54" t="n">
         <v>58</v>
@@ -7236,7 +7314,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C55" t="n">
         <v>57</v>
@@ -7269,7 +7347,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C56" t="n">
         <v>56</v>
@@ -7294,7 +7372,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C57" t="n">
         <v>56</v>
@@ -7319,7 +7397,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C58" t="n">
         <v>55</v>
@@ -7369,7 +7447,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C60" t="n">
         <v>53</v>
@@ -7394,7 +7472,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C61" t="n">
         <v>53</v>
@@ -7494,7 +7572,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C65" t="n">
         <v>51</v>
@@ -7519,7 +7597,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C66" t="n">
         <v>51</v>
@@ -7619,7 +7697,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C70" t="n">
         <v>49</v>
@@ -7644,7 +7722,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C71" t="n">
         <v>49</v>
@@ -7669,7 +7747,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C72" t="n">
         <v>49</v>
@@ -7694,7 +7772,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C73" t="n">
         <v>49</v>
@@ -7719,7 +7797,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C74" t="n">
         <v>49</v>
@@ -7744,7 +7822,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C75" t="n">
         <v>49</v>
@@ -7844,7 +7922,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C79" t="n">
         <v>49</v>
@@ -7869,7 +7947,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C80" t="n">
         <v>49</v>
@@ -8294,7 +8372,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C97" t="n">
         <v>46</v>
@@ -8344,7 +8422,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C99" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-06 12:56 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$127</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1610,54 +1610,50 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="n">
         <v>78</v>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Praktikum Trade Marketing (m/w/d)</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="F25" t="n">
         <v>6</v>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5910613503?se=WhIwK-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65AC17FF771A1B5B902EFA529296A7E02B52E694</t>
         </is>
@@ -1904,25 +1900,25 @@
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
@@ -1943,33 +1939,31 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>2</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
@@ -1978,7 +1972,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1989,28 +1983,28 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -2022,7 +2016,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2033,7 +2027,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2044,17 +2038,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Brand Management – Gum &amp; Chocolate Portfolios</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -2066,7 +2060,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2077,7 +2071,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5806012633?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2092,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -2110,7 +2104,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2121,31 +2115,33 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>6</v>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
@@ -2154,7 +2150,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2165,7 +2161,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2177,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2211,7 +2207,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2223,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2238,7 +2234,11 @@
       <c r="F38" t="n">
         <v>6</v>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2257,7 +2257,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,23 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>6</v>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2307,7 +2303,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2540,48 +2536,44 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="n">
         <v>62</v>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>BILD</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Praktikum Business Development (Video)</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Berlin, Deutschland</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5911182062?se=Fl00L-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=53169F7FEF5F866C5881E6837F4AEA357B701A1A</t>
         </is>
@@ -3654,48 +3646,44 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="n">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="n">
         <v>54</v>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>The BIG Jobsite</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr">
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5909334573?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -3986,7 +3974,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3998,7 +3986,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4020,7 +4008,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4030,7 +4018,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4042,7 +4030,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4053,7 +4041,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4062,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4097,7 +4085,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4106,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4130,7 +4118,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4141,7 +4129,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4150,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4185,7 +4173,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
+          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4194,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Pempelfort, Düsseldorf</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4229,7 +4217,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
+          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4238,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pempelfort, Düsseldorf</t>
+          <t>Neustadt, Hamburg</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4273,7 +4261,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
+          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
         </is>
       </c>
     </row>
@@ -4284,21 +4272,25 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Neustadt, Hamburg</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H84" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4306,7 +4298,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4317,7 +4309,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4328,25 +4320,21 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4365,7 +4353,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4376,17 +4364,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4398,7 +4386,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4409,28 +4397,28 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4442,7 +4430,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4453,7 +4441,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -4464,29 +4452,29 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4497,7 +4485,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4501,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4530,7 +4518,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4541,40 +4529,40 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4585,7 +4573,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4596,25 +4584,29 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; Campaign Management (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4625,7 +4617,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-campaign-management-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4636,19 +4628,15 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
@@ -4658,7 +4646,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4669,7 +4657,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4680,19 +4668,15 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Unterbilk, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
@@ -4702,7 +4686,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4713,7 +4697,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -4729,7 +4713,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Skincare Merchandising Intern</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -4742,7 +4726,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4753,7 +4737,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4769,7 +4753,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
+          <t>Internship / Trade Marketing Europe</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -4782,7 +4766,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4793,7 +4777,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
         </is>
       </c>
     </row>
@@ -4809,7 +4793,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
+          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -4822,7 +4806,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4833,7 +4817,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
         </is>
       </c>
     </row>
@@ -4849,7 +4833,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Internship / Trade Marketing Europe</t>
+          <t>Internship / Skincare Merchandising</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -4873,7 +4857,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4873,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
+          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -4902,7 +4886,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4913,7 +4897,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
+          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
         </is>
       </c>
     </row>
@@ -4924,15 +4908,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Internship / Skincare Merchandising</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr"/>
+          <t>Praktikum Category Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Münster, Nordrhein-Westfalen</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
@@ -4942,7 +4930,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4953,7 +4941,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4964,15 +4952,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr"/>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
@@ -4982,7 +4974,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4993,7 +4985,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5004,17 +4996,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5026,7 +5018,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5037,7 +5029,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5048,29 +5040,29 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5081,7 +5073,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -5092,17 +5084,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5125,7 +5117,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5136,29 +5128,29 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5169,7 +5161,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
         </is>
       </c>
     </row>
@@ -5180,29 +5172,29 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5213,7 +5205,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
         </is>
       </c>
     </row>
@@ -5224,29 +5216,29 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Brand Manager Intern - Nestlé Baby</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5257,7 +5249,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
         </is>
       </c>
     </row>
@@ -5273,7 +5265,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
+          <t>Brand Manager Intern - Nutrition</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5290,7 +5282,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5301,7 +5293,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5309,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nestlé Baby</t>
+          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5334,7 +5326,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5345,7 +5337,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5353,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nutrition</t>
+          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5378,7 +5370,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -5389,7 +5381,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
         </is>
       </c>
     </row>
@@ -5400,29 +5392,29 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -5433,7 +5425,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -5444,29 +5436,29 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5477,7 +5469,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -5488,17 +5480,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5521,7 +5513,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5532,17 +5524,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5554,7 +5546,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -5565,7 +5557,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5576,17 +5568,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Rankweil, Feldkirch</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5598,7 +5590,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -5609,7 +5601,7 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/land/ad/5896357793?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA0A29D7B49D4A241A4DCD6CB490D5AA41F3E792</t>
         </is>
       </c>
     </row>
@@ -5620,17 +5612,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Marketing (all genders)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Heidelberg, Baden-Württemberg</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5642,7 +5634,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -5653,7 +5645,7 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5664,17 +5656,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
+          <t>Samedo GmbH</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikum (m/w/d) - E-Commerce</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Rankweil, Feldkirch</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5686,7 +5678,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5697,7 +5689,7 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5896357793?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA0A29D7B49D4A241A4DCD6CB490D5AA41F3E792</t>
+          <t>https://www.adzuna.de/details/5910171389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5708,17 +5700,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Reckitt</t>
+          <t>Samedo GmbH</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (all genders)</t>
+          <t>Praktikum (m/w/d) - E-Commerce</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Heidelberg, Baden-Württemberg</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5730,7 +5722,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5741,124 +5733,116 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5910608498?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>Samedo GmbH</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum (m/w/d) - E-Commerce</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="inlineStr"/>
-      <c r="G118" s="2" t="inlineStr"/>
-      <c r="H118" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I118" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="J118" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K118" s="2" t="inlineStr"/>
-      <c r="L118" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5910171389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A118" t="inlineStr"/>
+      <c r="B118" t="n">
+        <v>48</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Paris, Paris, France</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>Samedo GmbH</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum (m/w/d) - E-Commerce</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>Altstadt-Lehel, München</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="inlineStr"/>
-      <c r="G119" s="2" t="inlineStr"/>
-      <c r="H119" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I119" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="J119" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K119" s="2" t="inlineStr"/>
-      <c r="L119" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5910608498?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="n">
+        <v>46</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>SUPA - Sport Und Party App</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Business Development Praktikum</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr"/>
       <c r="B120" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Paris, Paris, France</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5870,7 +5854,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -5881,28 +5865,28 @@
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr"/>
       <c r="B121" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5914,7 +5898,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -5925,28 +5909,28 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr"/>
       <c r="B122" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5969,7 +5953,7 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5980,17 +5964,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -6002,7 +5986,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -6013,7 +5997,7 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6018,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -6057,7 +6041,7 @@
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6078,7 +6062,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -6101,7 +6085,7 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6112,17 +6096,17 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -6145,7 +6129,7 @@
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6156,12 +6140,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6189,100 +6173,12 @@
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr"/>
-      <c r="B128" t="n">
-        <v>45</v>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr"/>
-      <c r="B129" t="n">
-        <v>45</v>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L129"/>
+  <autoFilter ref="A1:L127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6349,7 +6245,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6374,7 +6270,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6399,7 +6295,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" t="n">
         <v>107</v>
@@ -6474,7 +6370,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
         <v>91</v>
@@ -6499,7 +6395,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -6557,7 +6453,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
         <v>89</v>
@@ -6582,7 +6478,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" t="n">
         <v>89</v>
@@ -6632,7 +6528,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" t="n">
         <v>89</v>
@@ -6665,7 +6561,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C14" t="n">
         <v>87</v>
@@ -6698,7 +6594,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C15" t="n">
         <v>87</v>
@@ -6748,7 +6644,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6773,7 +6669,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -6806,7 +6702,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -6839,7 +6735,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
@@ -6864,7 +6760,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C21" t="n">
         <v>84</v>
@@ -6889,7 +6785,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C22" t="n">
         <v>84</v>
@@ -6914,7 +6810,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C23" t="n">
         <v>84</v>
@@ -6939,7 +6835,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C24" t="n">
         <v>84</v>
@@ -7014,7 +6910,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C27" t="n">
         <v>83</v>
@@ -7122,7 +7018,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C31" t="n">
         <v>78</v>
@@ -7147,7 +7043,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C32" t="n">
         <v>78</v>
@@ -7172,7 +7068,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C33" t="n">
         <v>77</v>
@@ -7197,7 +7093,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C34" t="n">
         <v>77</v>
@@ -7297,7 +7193,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C38" t="n">
         <v>73</v>
@@ -7322,7 +7218,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C39" t="n">
         <v>73</v>
@@ -7380,7 +7276,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C41" t="n">
         <v>72</v>
@@ -7405,7 +7301,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C42" t="n">
         <v>72</v>
@@ -7480,7 +7376,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C45" t="n">
         <v>68</v>
@@ -7555,7 +7451,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C48" t="n">
         <v>65</v>
@@ -7580,7 +7476,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C49" t="n">
         <v>64</v>
@@ -7605,7 +7501,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C50" t="n">
         <v>64</v>
@@ -7630,7 +7526,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C51" t="n">
         <v>62</v>
@@ -7655,7 +7551,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C52" t="n">
         <v>62</v>
@@ -7680,7 +7576,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C53" t="n">
         <v>62</v>
@@ -7705,7 +7601,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C54" t="n">
         <v>60</v>
@@ -7763,7 +7659,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C56" t="n">
         <v>59</v>
@@ -7813,7 +7709,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C58" t="n">
         <v>57</v>
@@ -7846,7 +7742,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C59" t="n">
         <v>56</v>
@@ -7871,7 +7767,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="C60" t="n">
         <v>56</v>
@@ -7896,7 +7792,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C61" t="n">
         <v>55</v>
@@ -7946,7 +7842,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C63" t="n">
         <v>53</v>
@@ -7971,7 +7867,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C64" t="n">
         <v>53</v>
@@ -8071,7 +7967,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C68" t="n">
         <v>51</v>
@@ -8096,7 +7992,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C69" t="n">
         <v>51</v>
@@ -8196,7 +8092,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C73" t="n">
         <v>49</v>
@@ -8221,7 +8117,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C74" t="n">
         <v>49</v>
@@ -8246,7 +8142,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C75" t="n">
         <v>49</v>
@@ -8271,7 +8167,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C76" t="n">
         <v>49</v>
@@ -8321,7 +8217,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C78" t="n">
         <v>49</v>
@@ -8346,7 +8242,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C79" t="n">
         <v>49</v>
@@ -8421,7 +8317,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C82" t="n">
         <v>49</v>
@@ -8471,7 +8367,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C84" t="n">
         <v>49</v>
@@ -8896,7 +8792,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C101" t="n">
         <v>46</v>
@@ -8946,7 +8842,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C103" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-09 12:46 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -566,27 +566,31 @@
     <row r="3">
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Düsseldorf</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
+          <t>Associate Product Marketing Manager BS/MS Intern, 2027</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Landstraße, Wien</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -594,7 +598,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -605,7 +609,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5912254007?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -616,7 +620,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Österreich</t>
+          <t>Peek &amp; Cloppenburg Düsseldorf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -626,7 +630,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Innere Stadt, Wien</t>
+          <t>Landstraße, Wien</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -640,7 +644,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -651,7 +655,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
+          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -672,7 +676,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Innere Stadt, Wien</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -686,7 +690,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -697,32 +701,32 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
+          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ABRIO GmbH</t>
+          <t>Peek &amp; Cloppenburg Österreich</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bockenheim, Frankfurt am Main</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
@@ -732,7 +736,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -743,7 +747,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
         </is>
       </c>
     </row>
@@ -754,25 +758,23 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>ABRIO GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
+          <t>Bockenheim, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -791,23 +793,23 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -815,10 +817,12 @@
           <t>München, München (Kreis)</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -826,7 +830,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -837,7 +841,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -848,17 +852,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -883,7 +887,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -894,21 +898,21 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing &amp; Brand Communication bei YSL (Luxe Division) - Start Mai für 6 Monate</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -918,7 +922,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -929,7 +933,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5899340175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -940,27 +944,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing &amp; Brand Communication bei YSL (Luxe Division) - Start Mai für 6 Monate</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -968,7 +968,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -979,7 +979,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5899340175?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -990,17 +990,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1029,7 +1029,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1040,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1058,17 +1058,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1079,7 +1079,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1090,31 +1090,35 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1125,7 +1129,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -1136,17 +1140,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1160,7 +1164,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1171,7 +1175,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1196,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1217,105 +1221,101 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>84</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Picnic</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Category Management Praktikum (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B18" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>PAIDAI GmbH</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Praktikum Product Marketing und Projektmanagement (m/w/d)</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>HafenCity, Hamburg</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5913315703?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="n">
-        <v>78</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Ferrero</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1342,7 +1342,11 @@
       <c r="F19" t="n">
         <v>6</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1361,7 +1365,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1372,17 +1376,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1396,7 +1400,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1407,7 +1411,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1418,27 +1422,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab Februar/März/April für 6 Monate</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>6</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2027-04-01</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1457,7 +1457,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5897975480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab Februar/März/April für 6 Monate</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-04-01</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1507,7 +1507,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5897975480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1557,7 +1557,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5910613503?se=WhIwK-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65AC17FF771A1B5B902EFA529296A7E02B52E694</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1591,12 +1591,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1607,28 +1607,28 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
+          <t>https://www.adzuna.de/land/ad/5910613503?se=WhIwK-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65AC17FF771A1B5B902EFA529296A7E02B52E694</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
+          <t>Praktikum Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1636,12 +1636,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1657,7 +1657,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1707,32 +1707,38 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1740,7 +1746,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1751,7 +1757,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1762,17 +1768,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1784,7 +1790,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1795,38 +1801,32 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Associate Product Marketing Manager BS/MS Intern, 2027</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>6</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2027-07-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1845,7 +1845,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5912254007?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
@@ -2032,46 +2032,50 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="n">
-        <v>69</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>The BIG Jobsite</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5918345837?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2082,29 +2086,29 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) Retail &amp; Trade Marketing</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Duesseldorf, DE</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2115,7 +2119,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Duesseldorf-Praktikant-%28mwd%29-Retail-&amp;-Trade-Marketing/1443408333/</t>
+          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
         </is>
       </c>
     </row>
@@ -2126,29 +2130,29 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikant (m/w/d) Retail &amp; Trade Marketing</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Duesseldorf, DE</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2159,7 +2163,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://jobdetails.nestle.com/job/Duesseldorf-Praktikant-%28mwd%29-Retail-&amp;-Trade-Marketing/1443408333/</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2184,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2192,7 +2196,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2203,38 +2207,32 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>6</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2242,7 +2240,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2253,7 +2251,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
@@ -2264,23 +2262,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>6</v>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2299,7 +2301,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2310,27 +2312,23 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>6</v>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2349,7 +2347,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2360,23 +2358,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F41" t="n">
         <v>6</v>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2395,31 +2397,33 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
@@ -2428,7 +2432,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2439,40 +2443,40 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5908496995?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2483,7 +2487,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5908496995?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2503,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing Royal Canin</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2516,7 +2520,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2538,29 +2542,29 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Internship in Trade Marketing Royal Canin</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2571,28 +2575,28 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5908264156?se=JEFAPRq_8RGTyvTH5qRQ7A&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=61DB8B099FEF69C3B9112B9C8897496D19A6BA45</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BILD</t>
+          <t>The BIG Jobsite</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Video)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2604,7 +2608,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2615,7 +2619,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5911182062?se=Fl00L-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=53169F7FEF5F866C5881E6837F4AEA357B701A1A</t>
+          <t>https://www.adzuna.de/land/ad/5908264156?se=JEFAPRq_8RGTyvTH5qRQ7A&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=61DB8B099FEF69C3B9112B9C8897496D19A6BA45</t>
         </is>
       </c>
     </row>
@@ -2626,12 +2630,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>BILD</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Business Development (Video)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2648,7 +2652,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2659,7 +2663,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5911182062?se=Fl00L-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=53169F7FEF5F866C5881E6837F4AEA357B701A1A</t>
         </is>
       </c>
     </row>
@@ -2670,17 +2674,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2703,7 +2707,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2723,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2736,7 +2740,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2747,7 +2751,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2767,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2780,7 +2784,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2791,7 +2795,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2802,17 +2806,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2824,7 +2828,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2835,7 +2839,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2860,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2879,38 +2883,32 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Aumovio</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development und Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Regensburg, Regensburg (Kreis)</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>6</v>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>2027-03-01</t>
-        </is>
-      </c>
+          <t>Wedding, Berlin</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2918,7 +2916,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2929,32 +2927,38 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5894317981?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Aumovio</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum - Business Development und Marketing</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+          <t>Regensburg, Regensburg (Kreis)</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>6</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2962,7 +2966,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2973,40 +2977,40 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/details/5894317981?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3017,40 +3021,40 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3061,7 +3065,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -3072,12 +3076,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3094,7 +3098,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3105,7 +3109,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3130,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -3149,26 +3153,30 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr"/>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
@@ -3178,7 +3186,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3189,7 +3197,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3200,22 +3208,16 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>6</v>
-      </c>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3224,7 +3226,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3235,7 +3237,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -3246,29 +3248,31 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SINGAPORE</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>6</v>
+      </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3279,7 +3283,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3290,31 +3294,29 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F62" t="n">
-        <v>6</v>
-      </c>
+          <t>SINGAPORE</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3325,31 +3327,33 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>6</v>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
@@ -3369,7 +3373,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3380,17 +3384,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -3413,7 +3417,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3433,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3437,9 +3441,7 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>6</v>
-      </c>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
@@ -3448,7 +3450,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3459,7 +3461,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3470,12 +3472,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3483,12 +3485,10 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="F66" t="n">
+        <v>6</v>
+      </c>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3507,7 +3507,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3518,24 +3518,28 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3551,7 +3555,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3571,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3584,7 +3588,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3595,7 +3599,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3606,29 +3610,29 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3639,23 +3643,23 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5909334573?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>BILD</t>
+          <t>The BIG Jobsite</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (video)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3672,7 +3676,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3683,7 +3687,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5911633064?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5909334573?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3694,29 +3698,29 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>BILD</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Business Development (video)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3727,7 +3731,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5911633064?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3738,29 +3742,29 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3771,7 +3775,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3782,12 +3786,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3804,7 +3808,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3815,28 +3819,28 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>AUTO1 Group</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3848,7 +3852,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3859,7 +3863,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
@@ -3870,17 +3874,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>AUTO1 Group</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3892,7 +3896,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3903,7 +3907,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3914,17 +3918,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3936,7 +3940,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3947,7 +3951,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3962,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3968,7 +3972,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3980,7 +3984,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3991,7 +3995,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4012,7 +4016,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4035,7 +4039,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4060,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4068,7 +4072,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4079,7 +4083,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -4100,7 +4104,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4123,7 +4127,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
+          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
         </is>
       </c>
     </row>
@@ -4144,7 +4148,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pempelfort, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4167,7 +4171,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
+          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4192,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Neustadt, Hamburg</t>
+          <t>Pempelfort, Düsseldorf</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4211,7 +4215,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
+          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
         </is>
       </c>
     </row>
@@ -4222,25 +4226,21 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Neustadt, Hamburg</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4259,7 +4259,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
         </is>
       </c>
     </row>
@@ -4270,21 +4270,25 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H84" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4303,7 +4307,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4314,17 +4318,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4336,7 +4340,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4347,28 +4351,28 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4380,7 +4384,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4391,7 +4395,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4402,29 +4406,29 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4435,7 +4439,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4455,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4468,7 +4472,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4479,40 +4483,40 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4523,7 +4527,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4548,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4556,7 +4560,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4567,7 +4571,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4578,17 +4582,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4600,7 +4604,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4611,7 +4615,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4622,15 +4626,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
@@ -4640,7 +4648,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4651,7 +4659,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4675,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -4691,7 +4699,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4707,7 +4715,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Skincare Merchandising Intern</t>
+          <t>Operational Trade Marketing Intern</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -4720,7 +4728,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4731,7 +4739,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Skincare-Merchandising-Intern-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -6239,7 +6247,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6264,7 +6272,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6289,7 +6297,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" t="n">
         <v>107</v>
@@ -6364,7 +6372,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
         <v>91</v>
@@ -6389,7 +6397,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C8" t="n">
         <v>89</v>
@@ -6447,7 +6455,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C10" t="n">
         <v>89</v>
@@ -6472,7 +6480,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" t="n">
         <v>89</v>
@@ -6497,7 +6505,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12" t="n">
         <v>89</v>
@@ -6555,7 +6563,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" t="n">
         <v>87</v>
@@ -6588,7 +6596,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C15" t="n">
         <v>87</v>
@@ -6609,7 +6617,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -6620,7 +6628,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -6634,18 +6642,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -6663,7 +6671,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -6729,7 +6737,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
@@ -6754,7 +6762,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C21" t="n">
         <v>84</v>
@@ -6779,7 +6787,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C22" t="n">
         <v>84</v>
@@ -6804,7 +6812,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C23" t="n">
         <v>84</v>
@@ -6829,7 +6837,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C24" t="n">
         <v>84</v>
@@ -6962,7 +6970,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
         <v>80</v>
@@ -7037,7 +7045,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C32" t="n">
         <v>78</v>
@@ -7062,7 +7070,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C33" t="n">
         <v>78</v>
@@ -7087,7 +7095,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C34" t="n">
         <v>77</v>
@@ -7112,7 +7120,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C35" t="n">
         <v>77</v>
@@ -7212,7 +7220,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C39" t="n">
         <v>73</v>
@@ -7237,7 +7245,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C40" t="n">
         <v>73</v>
@@ -7295,7 +7303,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C42" t="n">
         <v>72</v>
@@ -7320,7 +7328,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C43" t="n">
         <v>72</v>
@@ -7341,118 +7349,118 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>The BIG Jobsite</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="C44" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C45" t="n">
         <v>69</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Groß- &amp; Einzelhandel Karriere</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C46" t="n">
         <v>69</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Groß- &amp; Einzelhandel Karriere</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C47" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="C48" t="n">
         <v>68</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -7466,18 +7474,18 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="C49" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -7491,18 +7499,18 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C50" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -7516,18 +7524,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C51" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -7541,25 +7549,25 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>7</v>
+        <v>70</v>
       </c>
       <c r="C52" t="n">
         <v>64</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -7570,7 +7578,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C53" t="n">
         <v>62</v>
@@ -7595,7 +7603,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C54" t="n">
         <v>62</v>
@@ -7620,7 +7628,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C55" t="n">
         <v>62</v>
@@ -7645,7 +7653,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C56" t="n">
         <v>60</v>
@@ -7728,7 +7736,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C59" t="n">
         <v>57</v>
@@ -7761,7 +7769,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C60" t="n">
         <v>56</v>
@@ -7786,7 +7794,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C61" t="n">
         <v>56</v>
@@ -7811,7 +7819,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C62" t="n">
         <v>55</v>
@@ -7861,7 +7869,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="C64" t="n">
         <v>53</v>
@@ -7886,7 +7894,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C65" t="n">
         <v>53</v>
@@ -8011,7 +8019,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C70" t="n">
         <v>51</v>
@@ -8036,7 +8044,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C71" t="n">
         <v>51</v>
@@ -8111,7 +8119,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C74" t="n">
         <v>49</v>
@@ -8136,7 +8144,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C75" t="n">
         <v>49</v>
@@ -8161,7 +8169,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C76" t="n">
         <v>49</v>
@@ -8186,7 +8194,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C77" t="n">
         <v>49</v>
@@ -8211,7 +8219,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C78" t="n">
         <v>49</v>
@@ -8261,7 +8269,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C80" t="n">
         <v>49</v>
@@ -8336,7 +8344,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C83" t="n">
         <v>49</v>
@@ -8361,7 +8369,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C84" t="n">
         <v>49</v>
@@ -8811,7 +8819,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C102" t="n">
         <v>46</v>
@@ -8836,7 +8844,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C103" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-14 11:22 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$127</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$120</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -518,21 +518,21 @@
     <row r="2">
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -548,7 +548,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -559,34 +559,36 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5895502880?se=EIPLzwe48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0668B6260348B06F79C79FBD16FB7D4160F27AC4</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Associate Product Marketing Manager BS/MS Intern, 2027</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>3</v>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-07-01</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -596,7 +598,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -607,38 +609,34 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502880?se=EIPLzwe48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0668B6260348B06F79C79FBD16FB7D4160F27AC4</t>
+          <t>https://www.adzuna.de/details/5912254007?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Associate Product Marketing Manager BS/MS Intern, 2027</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>3</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2027-07-01</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -646,7 +644,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -657,7 +655,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5912254007?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
         </is>
       </c>
     </row>
@@ -668,21 +666,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>Peek &amp; Cloppenburg Düsseldorf</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Landstraße, Wien</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
@@ -692,7 +690,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -703,7 +701,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
+          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -714,7 +712,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Düsseldorf</t>
+          <t>Peek &amp; Cloppenburg Österreich</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -724,7 +722,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Landstraße, Wien</t>
+          <t>Innere Stadt, Wien</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -738,7 +736,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -749,7 +747,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
         </is>
       </c>
     </row>
@@ -770,7 +768,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Innere Stadt, Wien</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -784,7 +782,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -795,32 +793,32 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
+          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Österreich</t>
+          <t>ABRIO GmbH</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
+          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Bockenheim, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
@@ -830,7 +828,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -841,7 +839,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
+          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -852,23 +850,25 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ABRIO GmbH</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bockenheim, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>München, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -887,7 +887,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1040,17 +1040,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1058,17 +1058,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1079,7 +1079,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1090,31 +1090,35 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1125,7 +1129,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -1136,17 +1140,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1160,7 +1164,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1171,7 +1175,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1196,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1217,31 +1221,33 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PAIDAI GmbH</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Product Marketing und Projektmanagement (m/w/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HafenCity, Hamburg</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
@@ -1250,7 +1256,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1261,38 +1267,32 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5913315703?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>PAIDAI GmbH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Product Marketing und Projektmanagement (m/w/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>HafenCity, Hamburg</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1311,7 +1311,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5913315703?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1338,7 +1338,11 @@
       <c r="F19" t="n">
         <v>6</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1357,7 +1361,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1368,17 +1372,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1392,7 +1396,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1403,7 +1407,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1414,27 +1418,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>6</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1453,7 +1453,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1503,7 +1503,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5910613503?se=WhIwK-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65AC17FF771A1B5B902EFA529296A7E02B52E694</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1537,12 +1537,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1553,28 +1553,28 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
+          <t>https://www.adzuna.de/land/ad/5910613503?se=WhIwK-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65AC17FF771A1B5B902EFA529296A7E02B52E694</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
+          <t>Praktikum Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1603,7 +1603,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1653,32 +1653,38 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>6</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1686,7 +1692,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1697,7 +1703,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2874,48 +2880,44 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="n">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="n">
         <v>59</v>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Germany, Hannover</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
         <is>
           <t>https://clarios.wd5.myworkdayjobs.com/clarioscareers/job/Germany-Hannover/Praktikant--m-w-d--im-Bereich-Trade-Marketing-DACH_WD49855</t>
         </is>
@@ -4294,48 +4296,44 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="n">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="n">
         <v>50</v>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Doctolib</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>IA Engineer intern (x/f/m) - Berlin</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E85" t="inlineStr">
         <is>
           <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" s="2" t="inlineStr"/>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I85" s="2" t="inlineStr">
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="J85" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K85" s="2" t="inlineStr"/>
-      <c r="L85" s="2" t="inlineStr">
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/doctolib/jobs/8015564003</t>
         </is>
@@ -5286,46 +5284,50 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr"/>
-      <c r="B108" t="n">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Nestle Deutschland</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Trade Marketing Intern - Purina</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Brussels, BE</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
         </is>
       </c>
     </row>
@@ -5336,17 +5338,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5369,7 +5371,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -5380,17 +5382,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5402,7 +5404,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -5413,7 +5415,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5424,17 +5426,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Rankweil, Feldkirch</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -5446,7 +5448,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5457,7 +5459,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5896357793?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA0A29D7B49D4A241A4DCD6CB490D5AA41F3E792</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5468,17 +5470,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Reckitt</t>
+          <t>RAUCH Fruchtsäfte GmbH &amp; Co OG</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (all genders)</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
+          <t>Rankweil, Feldkirch</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5490,7 +5492,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -5501,7 +5503,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/land/ad/5896357793?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA0A29D7B49D4A241A4DCD6CB490D5AA41F3E792</t>
         </is>
       </c>
     </row>
@@ -5512,17 +5514,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Samedo GmbH</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) - E-Commerce</t>
+          <t>Praktikum Brand Marketing (all genders)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5534,7 +5536,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -5545,7 +5547,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5910171389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5568,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5589,7 +5591,7 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5910608498?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5910171389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5600,17 +5602,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Samedo GmbH</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
+          <t>Praktikum (m/w/d) - E-Commerce</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5622,7 +5624,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -5633,28 +5635,28 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5910608498?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr"/>
       <c r="B116" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Paris, Paris, France</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5666,7 +5668,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5677,28 +5679,28 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
+          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
       <c r="B117" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Paris, Paris, France</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5710,7 +5712,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5721,7 +5723,7 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5744,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5765,99 +5767,99 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="n">
+        <v>46</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>SUPA - Sport Und Party App</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Business Development Praktikum</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Altstadt-Nord, Köln</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B119" s="2" t="n">
+      <c r="B120" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="C119" s="2" t="inlineStr">
+      <c r="C120" s="2" t="inlineStr">
         <is>
           <t>Deutsche Lufthansa AG</t>
         </is>
       </c>
-      <c r="D119" s="2" t="inlineStr">
+      <c r="D120" s="2" t="inlineStr">
         <is>
           <t>Praktikum im Bereich Business Development and Sustainability</t>
         </is>
       </c>
-      <c r="E119" s="2" t="inlineStr">
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
-      <c r="F119" s="2" t="inlineStr"/>
-      <c r="G119" s="2" t="inlineStr"/>
-      <c r="H119" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I119" s="2" t="inlineStr">
+      <c r="F120" s="2" t="inlineStr"/>
+      <c r="G120" s="2" t="inlineStr"/>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="J119" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K119" s="2" t="inlineStr"/>
-      <c r="L119" s="2" t="inlineStr">
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K120" s="2" t="inlineStr"/>
+      <c r="L120" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr"/>
-      <c r="B120" t="n">
-        <v>45</v>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Helu.io GmbH</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Margareten, Wien</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5868,17 +5870,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5890,7 +5892,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -5901,7 +5903,7 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5917,7 +5919,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5945,7 +5947,7 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5961,12 +5963,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -5989,7 +5991,7 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6005,7 +6007,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6033,7 +6035,7 @@
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6044,17 +6046,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -6077,7 +6079,7 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6100,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -6121,12 +6123,56 @@
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr"/>
+      <c r="B127" t="n">
+        <v>45</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L126"/>
+  <autoFilter ref="A1:L127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6193,7 +6239,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6218,7 +6264,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6243,7 +6289,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" t="n">
         <v>107</v>
@@ -6268,7 +6314,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" t="n">
         <v>105</v>
@@ -6326,7 +6372,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="C7" t="n">
         <v>97</v>
@@ -6359,7 +6405,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C8" t="n">
         <v>91</v>
@@ -6384,7 +6430,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" t="n">
         <v>91</v>
@@ -6409,7 +6455,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C10" t="n">
         <v>89</v>
@@ -6459,7 +6505,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C12" t="n">
         <v>89</v>
@@ -6509,7 +6555,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C14" t="n">
         <v>89</v>
@@ -6567,7 +6613,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C16" t="n">
         <v>87</v>
@@ -6592,7 +6638,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6642,7 +6688,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -6675,7 +6721,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
@@ -6708,7 +6754,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C21" t="n">
         <v>84</v>
@@ -6733,7 +6779,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C22" t="n">
         <v>84</v>
@@ -6758,7 +6804,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C23" t="n">
         <v>84</v>
@@ -6783,7 +6829,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C24" t="n">
         <v>84</v>
@@ -6808,7 +6854,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" t="n">
         <v>84</v>
@@ -6941,7 +6987,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C30" t="n">
         <v>80</v>
@@ -7016,7 +7062,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C33" t="n">
         <v>78</v>
@@ -7041,7 +7087,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C34" t="n">
         <v>78</v>
@@ -7066,7 +7112,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C35" t="n">
         <v>78</v>
@@ -7091,7 +7137,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C36" t="n">
         <v>77</v>
@@ -7116,7 +7162,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C37" t="n">
         <v>77</v>
@@ -7216,7 +7262,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C41" t="n">
         <v>73</v>
@@ -7241,7 +7287,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C42" t="n">
         <v>73</v>
@@ -7266,7 +7312,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C43" t="n">
         <v>73</v>
@@ -7299,7 +7345,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C44" t="n">
         <v>72</v>
@@ -7324,7 +7370,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C45" t="n">
         <v>72</v>
@@ -7349,7 +7395,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C46" t="n">
         <v>70</v>
@@ -7382,7 +7428,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C47" t="n">
         <v>70</v>
@@ -7415,7 +7461,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C48" t="n">
         <v>70</v>
@@ -7440,7 +7486,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C49" t="n">
         <v>69</v>
@@ -7615,7 +7661,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C56" t="n">
         <v>66</v>
@@ -7640,7 +7686,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C57" t="n">
         <v>65</v>
@@ -7665,7 +7711,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C58" t="n">
         <v>64</v>
@@ -7690,7 +7736,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C59" t="n">
         <v>62</v>
@@ -7715,7 +7761,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C60" t="n">
         <v>62</v>
@@ -7740,7 +7786,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C61" t="n">
         <v>62</v>
@@ -7765,7 +7811,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C62" t="n">
         <v>60</v>
@@ -7798,7 +7844,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C63" t="n">
         <v>59</v>
@@ -7823,7 +7869,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C64" t="n">
         <v>59</v>
@@ -7848,7 +7894,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C65" t="n">
         <v>58</v>
@@ -7873,7 +7919,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C66" t="n">
         <v>57</v>
@@ -7906,7 +7952,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C67" t="n">
         <v>56</v>
@@ -7931,7 +7977,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C68" t="n">
         <v>55</v>
@@ -7981,7 +8027,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C70" t="n">
         <v>53</v>
@@ -8006,7 +8052,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C71" t="n">
         <v>53</v>
@@ -8106,7 +8152,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C75" t="n">
         <v>51</v>
@@ -8156,7 +8202,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C77" t="n">
         <v>51</v>
@@ -8231,7 +8277,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C80" t="n">
         <v>49</v>
@@ -8256,7 +8302,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C81" t="n">
         <v>49</v>
@@ -8806,7 +8852,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C103" t="n">
         <v>46</v>
@@ -8856,7 +8902,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C105" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-16 10:53 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$120</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -942,17 +942,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -960,7 +960,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -981,7 +981,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -992,12 +992,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1010,17 +1010,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1031,7 +1031,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1047,18 +1047,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) Retail &amp; Trade Marketing</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Duesseldorf, DE</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>fmcg</t>
@@ -1066,7 +1070,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1077,7 +1081,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Duesseldorf-Praktikant-%28mwd%29-Retail-&amp;-Trade-Marketing/1443408333/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1148,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1169,31 +1173,33 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PAIDAI GmbH</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Product Marketing und Projektmanagement (m/w/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HafenCity, Hamburg</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>6</v>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
@@ -1202,7 +1208,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1213,38 +1219,32 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5913315703?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>PAIDAI GmbH</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Product Marketing und Projektmanagement (m/w/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>HafenCity, Hamburg</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1263,7 +1263,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5913315703?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1290,7 +1290,11 @@
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1309,7 +1313,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1320,17 +1324,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1344,7 +1348,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1355,7 +1359,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1366,27 +1370,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>6</v>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1405,7 +1405,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1455,7 +1455,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5910613503?se=WhIwK-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65AC17FF771A1B5B902EFA529296A7E02B52E694</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1489,12 +1489,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1505,28 +1505,28 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
+          <t>https://www.adzuna.de/land/ad/5910613503?se=WhIwK-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65AC17FF771A1B5B902EFA529296A7E02B52E694</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
+          <t>Praktikum Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1555,7 +1555,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Trade-Marketing-%28mwd%29-60329/1440823833/</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1605,32 +1605,38 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5895255365?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – Feb/März 2027</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1638,7 +1644,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1649,7 +1655,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5897088508?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2020,29 +2026,29 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikant (m/w/d) Retail &amp; Trade Marketing</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Duesseldorf, DE</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2053,7 +2059,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://jobdetails.nestle.com/job/Duesseldorf-Praktikant-%28mwd%29-Retail-&amp;-Trade-Marketing/1443408333/</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2080,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -2086,7 +2092,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2097,7 +2103,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -2108,17 +2114,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2130,7 +2136,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2141,38 +2147,32 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>The BIG Jobsite</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>6</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2191,7 +2191,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5908264156?se=JEFAPRq_8RGTyvTH5qRQ7A&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=61DB8B099FEF69C3B9112B9C8897496D19A6BA45</t>
         </is>
       </c>
     </row>
@@ -2202,17 +2202,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2241,7 +2241,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2252,23 +2252,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>6</v>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2287,31 +2291,33 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>6</v>
+      </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
@@ -2320,7 +2326,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2331,40 +2337,40 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5908496995?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing Royal Canin</t>
+          <t>Praktikum Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2375,7 +2381,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5908496995?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2386,29 +2392,29 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Internship in Trade Marketing Royal Canin</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2419,7 +2425,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5908264156?se=JEFAPRq_8RGTyvTH5qRQ7A&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=61DB8B099FEF69C3B9112B9C8897496D19A6BA45</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
@@ -2828,21 +2834,21 @@
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2854,7 +2860,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2865,7 +2871,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2892,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2909,30 +2915,26 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
@@ -2942,7 +2944,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2953,7 +2955,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -2964,16 +2966,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
+          <t>Praktikum - Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>6</v>
+      </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
@@ -2982,7 +2990,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2993,7 +3001,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3004,31 +3012,29 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>6</v>
-      </c>
+          <t>SINGAPORE</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3039,7 +3045,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
         </is>
       </c>
     </row>
@@ -3050,29 +3056,31 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SINGAPORE</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>6</v>
+      </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3083,33 +3091,31 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>6</v>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3129,7 +3135,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3140,17 +3146,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -3173,7 +3179,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3195,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3197,7 +3203,9 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="n">
+        <v>6</v>
+      </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3206,7 +3214,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3217,101 +3225,103 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
-      <c r="B61" t="n">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food - ['Vollzeit']</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>6</v>
-      </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5929202857?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="n">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Marc O'Polo</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Lidl Stiftung &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie - ['Vollzeit']</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5929202866?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3322,24 +3332,28 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3355,7 +3369,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3385,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3388,7 +3402,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3399,7 +3413,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3410,29 +3424,29 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3443,7 +3457,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5909334573?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
@@ -3459,7 +3473,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3476,7 +3490,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3487,103 +3501,103 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5909334573?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="n">
+        <v>54</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>The BIG Jobsite</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5922303195?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B67" s="2" t="n">
+      <c r="B68" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>Doctolib</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>Praktikum Public Affairs &amp; Advocacy (x/f/m)</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr"/>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>2027-01-01</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr"/>
-      <c r="L67" s="2" t="inlineStr">
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/doctolib/jobs/8026774003</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr"/>
-      <c r="B68" t="n">
-        <v>52</v>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>BILD</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (video)</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5911633064?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3594,12 +3608,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>BILD</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Business Development (video)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3616,7 +3630,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3627,7 +3641,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5911633064?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3638,12 +3652,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3660,7 +3674,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3671,28 +3685,28 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>AUTO1 Group</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3704,7 +3718,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3715,7 +3729,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
@@ -3726,17 +3740,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CHECK24 Vergleichsportal</t>
+          <t>AUTO1 Group</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Shopping</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -3748,7 +3762,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3759,7 +3773,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3770,17 +3784,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>CHECK24 Vergleichsportal</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development – Shopping</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3792,7 +3806,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3803,7 +3817,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5875663104?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3828,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3824,7 +3838,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3836,7 +3850,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3847,7 +3861,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3882,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3891,7 +3905,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3926,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3924,7 +3938,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3935,7 +3949,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -3956,7 +3970,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3979,7 +3993,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
+          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4014,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pempelfort, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4023,7 +4037,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
+          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4058,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Neustadt, Hamburg</t>
+          <t>Pempelfort, Düsseldorf</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4067,7 +4081,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
+          <t>https://www.adzuna.de/land/ad/5894022404?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8AA10F41BDD52042E79750491C8CC3B2BC84AEEF</t>
         </is>
       </c>
     </row>
@@ -4078,25 +4092,21 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Neustadt, Hamburg</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4104,7 +4114,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4115,7 +4125,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
         </is>
       </c>
     </row>
@@ -4126,21 +4136,25 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H81" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4159,7 +4173,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4170,17 +4184,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4192,7 +4206,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4203,28 +4217,28 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>IA Engineer intern (x/f/m) - Berlin</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4236,7 +4250,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4247,7 +4261,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/8015564003</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4258,29 +4272,29 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>IA Engineer intern (x/f/m) - Berlin</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4291,7 +4305,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/8015564003</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4321,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4324,7 +4338,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4335,40 +4349,40 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4379,7 +4393,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4414,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4412,7 +4426,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4423,7 +4437,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4434,17 +4448,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4456,7 +4470,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4467,7 +4481,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4478,15 +4492,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -4496,7 +4514,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4507,7 +4525,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4523,7 +4541,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -4547,7 +4565,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4581,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Internship / Trade Marketing Europe</t>
+          <t>Operational Trade Marketing Intern</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -4576,7 +4594,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4587,7 +4605,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4621,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
+          <t>Internship / Trade Marketing Europe</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -4627,7 +4645,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
         </is>
       </c>
     </row>
@@ -4643,7 +4661,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Internship / Skincare Merchandising</t>
+          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -4667,7 +4685,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4701,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
+          <t>Internship / Skincare Merchandising</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -4696,7 +4714,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4707,7 +4725,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4718,19 +4736,15 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Münster, Nordrhein-Westfalen</t>
-        </is>
-      </c>
+          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
@@ -4740,7 +4754,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4751,51 +4765,51 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
-      <c r="B96" t="n">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Henkel</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Coty</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Internship/Trade Marketing Assitant</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.coty.com/job/Paris-InternshipTrade-Marketing-Assitant-J-75002/1448411633/</t>
         </is>
       </c>
     </row>
@@ -4806,17 +4820,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4828,7 +4842,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4839,7 +4853,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4850,29 +4864,29 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4883,7 +4897,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4894,17 +4908,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4927,7 +4941,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4938,29 +4952,29 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4971,7 +4985,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -4982,29 +4996,29 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5015,7 +5029,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5026,29 +5040,29 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nestlé Baby</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5059,7 +5073,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
+          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
         </is>
       </c>
     </row>
@@ -5075,7 +5089,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nutrition</t>
+          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5092,7 +5106,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5103,7 +5117,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
         </is>
       </c>
     </row>
@@ -5119,7 +5133,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
+          <t>Brand Manager Intern - Nestlé Baby</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5136,7 +5150,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5147,7 +5161,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5177,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
+          <t>Brand Manager Intern - Nutrition</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5180,7 +5194,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5191,55 +5205,51 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="n">
+      <c r="A106" t="inlineStr"/>
+      <c r="B106" t="n">
         <v>49</v>
       </c>
-      <c r="C106" s="2" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>Nestle Deutschland</t>
         </is>
       </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>Trade Marketing Intern - Purina</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
         <is>
           <t>Brussels, BE</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr"/>
-      <c r="G106" s="2" t="inlineStr"/>
-      <c r="H106" s="2" t="inlineStr">
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J106" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K106" s="2" t="inlineStr"/>
-      <c r="L106" s="2" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
         </is>
       </c>
     </row>
@@ -5250,29 +5260,29 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5283,7 +5293,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
         </is>
       </c>
     </row>
@@ -5294,29 +5304,29 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Trade Marketing Intern - Purina</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5327,7 +5337,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
         </is>
       </c>
     </row>
@@ -5338,17 +5348,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Reckitt</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (all genders)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5360,7 +5370,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -5371,7 +5381,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5382,17 +5392,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Samedo GmbH</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) - E-Commerce</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5404,7 +5414,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -5415,7 +5425,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5910171389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5426,17 +5436,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Samedo GmbH</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) - E-Commerce</t>
+          <t>Praktikum Brand Marketing (all genders)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -5448,7 +5458,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5459,7 +5469,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5910608498?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5470,17 +5480,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Samedo GmbH</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
+          <t>Praktikum (m/w/d) - E-Commerce</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5492,7 +5502,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -5503,28 +5513,28 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5910171389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr"/>
       <c r="B113" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Samedo GmbH</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
+          <t>Praktikum (m/w/d) - E-Commerce</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Paris, Paris, France</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5536,7 +5546,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -5547,28 +5557,28 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
+          <t>https://www.adzuna.de/details/5910608498?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr"/>
       <c r="B114" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5580,7 +5590,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -5591,28 +5601,28 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr"/>
       <c r="B115" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Stage - Chargé de campagne CRM B2B (x/f/m) - janvier 2027</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Paris, Paris, France</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5624,7 +5634,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -5635,28 +5645,28 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7993977003</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr"/>
       <c r="B116" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Deutsche Lufthansa AG</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development and Sustainability</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5668,7 +5678,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5679,28 +5689,28 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
       <c r="B117" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5712,7 +5722,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5723,7 +5733,7 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5734,17 +5744,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Deutsche Lufthansa AG</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum im Bereich Business Development and Sustainability</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5756,7 +5766,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -5767,7 +5777,7 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5778,17 +5788,17 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5800,7 +5810,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -5811,7 +5821,7 @@
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5842,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5855,7 +5865,7 @@
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5886,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5899,7 +5909,7 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5910,17 +5920,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5943,7 +5953,7 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5954,12 +5964,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5987,12 +5997,100 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr"/>
+      <c r="B124" t="n">
+        <v>45</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr"/>
+      <c r="B125" t="n">
+        <v>45</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L123"/>
+  <autoFilter ref="A1:L125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6059,7 +6157,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6084,7 +6182,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6109,7 +6207,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" t="n">
         <v>107</v>
@@ -6134,7 +6232,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" t="n">
         <v>105</v>
@@ -6192,7 +6290,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C7" t="n">
         <v>97</v>
@@ -6225,7 +6323,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C8" t="n">
         <v>91</v>
@@ -6250,7 +6348,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
         <v>91</v>
@@ -6275,7 +6373,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C10" t="n">
         <v>89</v>
@@ -6325,7 +6423,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C12" t="n">
         <v>89</v>
@@ -6375,7 +6473,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" t="n">
         <v>89</v>
@@ -6433,7 +6531,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C16" t="n">
         <v>87</v>
@@ -6458,7 +6556,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6508,7 +6606,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C19" t="n">
         <v>84</v>
@@ -6541,7 +6639,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
@@ -6574,7 +6672,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C21" t="n">
         <v>84</v>
@@ -6599,7 +6697,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C22" t="n">
         <v>84</v>
@@ -6624,7 +6722,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" t="n">
         <v>84</v>
@@ -6649,7 +6747,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C24" t="n">
         <v>84</v>
@@ -6674,7 +6772,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" t="n">
         <v>84</v>
@@ -6807,7 +6905,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C30" t="n">
         <v>80</v>
@@ -6882,7 +6980,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C33" t="n">
         <v>78</v>
@@ -6907,7 +7005,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C34" t="n">
         <v>78</v>
@@ -6932,7 +7030,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C35" t="n">
         <v>78</v>
@@ -6957,7 +7055,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C36" t="n">
         <v>77</v>
@@ -6982,7 +7080,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C37" t="n">
         <v>77</v>
@@ -7082,7 +7180,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C41" t="n">
         <v>73</v>
@@ -7107,7 +7205,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C42" t="n">
         <v>73</v>
@@ -7132,7 +7230,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C43" t="n">
         <v>73</v>
@@ -7165,7 +7263,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C44" t="n">
         <v>72</v>
@@ -7190,7 +7288,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C45" t="n">
         <v>72</v>
@@ -7215,7 +7313,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C46" t="n">
         <v>70</v>
@@ -7248,7 +7346,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C47" t="n">
         <v>70</v>
@@ -7281,7 +7379,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C48" t="n">
         <v>70</v>
@@ -7306,7 +7404,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C49" t="n">
         <v>69</v>
@@ -7481,7 +7579,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C56" t="n">
         <v>66</v>
@@ -7506,7 +7604,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C57" t="n">
         <v>65</v>
@@ -7531,7 +7629,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C58" t="n">
         <v>64</v>
@@ -7552,50 +7650,50 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C59" t="n">
         <v>62</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C60" t="n">
         <v>62</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7729,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C62" t="n">
         <v>60</v>
@@ -7664,7 +7762,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C63" t="n">
         <v>59</v>
@@ -7689,7 +7787,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C64" t="n">
         <v>59</v>
@@ -7714,7 +7812,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C65" t="n">
         <v>58</v>
@@ -7739,7 +7837,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C66" t="n">
         <v>57</v>
@@ -7772,7 +7870,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C67" t="n">
         <v>56</v>
@@ -7797,7 +7895,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C68" t="n">
         <v>55</v>
@@ -7847,7 +7945,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C70" t="n">
         <v>53</v>
@@ -7872,7 +7970,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C71" t="n">
         <v>53</v>
@@ -7947,7 +8045,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C74" t="n">
         <v>51</v>
@@ -8022,7 +8120,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C77" t="n">
         <v>51</v>
@@ -8097,7 +8195,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C80" t="n">
         <v>49</v>
@@ -8122,7 +8220,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C81" t="n">
         <v>49</v>
@@ -8672,7 +8770,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C103" t="n">
         <v>46</v>
@@ -8722,7 +8820,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C105" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-19 12:19 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -518,29 +518,29 @@
     <row r="2">
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Associate Product Marketing Manager BS/MS Intern, 2027</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2027-07-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -561,34 +561,38 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5912254007?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Associate Product Marketing Manager BS/MS Intern, 2027</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>3</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -596,7 +600,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -607,7 +611,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
+          <t>https://www.adzuna.de/details/5912254007?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -618,21 +622,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Düsseldorf</t>
+          <t>ABRIO GmbH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
+          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Landstraße, Wien</t>
+          <t>Bockenheim, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
@@ -642,7 +646,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -653,7 +657,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -664,21 +668,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Österreich</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Innere Stadt, Wien</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
@@ -699,7 +703,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
+          <t>https://www.adzuna.de/land/ad/5893969437?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=052D5392382A8880129292F79681D8C750EAF3FD</t>
         </is>
       </c>
     </row>
@@ -710,7 +714,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg Österreich</t>
+          <t>Peek &amp; Cloppenburg Düsseldorf</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -720,7 +724,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Landstraße, Wien</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -745,32 +749,32 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
+          <t>https://www.adzuna.at/details/5895310424?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ABRIO GmbH</t>
+          <t>Peek &amp; Cloppenburg Österreich</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bockenheim, Frankfurt am Main</t>
+          <t>Innere Stadt, Wien</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
@@ -780,7 +784,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -791,36 +795,34 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/land/ad/5893983102?se=3Pib1Tu38RGSC5OxuzM0QA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0D8BB78FEA70CD33803247EDC45F9C8333EC0706</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>Peek &amp; Cloppenburg Österreich</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Brand Management &amp; Fashion PR (m/w/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
+          <t>Wien, Österreich</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -828,7 +830,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -839,82 +841,80 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
+          <t>https://www.adzuna.at/land/ad/5895447115?se=JKEK5ge48RG_dsLAqOI1yA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C3371E814C89C6E26AC0E52DE82C1EC2AD0532CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="n">
+        <v>87</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SERVICEPLAN Gruppe</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>München, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>qado GmbH</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Sales Development Representative (SDR) Praktikum / Werkstudium (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Altstadt-Lehel, München</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5930818508?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>qado GmbH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>Sales Development Representative (SDR) Praktikum / Werkstudium (m/w/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -935,7 +935,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5930818508?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -946,17 +946,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -981,7 +981,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -992,27 +992,23 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1020,7 +1016,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1031,7 +1027,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1042,17 +1038,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1060,7 +1056,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1070,7 +1066,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1081,7 +1077,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2664,18 +2660,20 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="n">
-        <v>6</v>
-      </c>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
@@ -2684,7 +2682,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2695,28 +2693,28 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2728,7 +2726,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2739,7 +2737,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2758,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2783,30 +2781,26 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
@@ -2816,7 +2810,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2827,7 +2821,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -5462,48 +5456,44 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="n">
+      <c r="A112" t="inlineStr"/>
+      <c r="B112" t="n">
         <v>48</v>
       </c>
-      <c r="C112" s="2" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>OBI Group Holding SE &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
         </is>
       </c>
-      <c r="E112" s="2" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>Wermelskirchen, Rheinisch-Bergischer Kreis</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr"/>
-      <c r="G112" s="2" t="inlineStr"/>
-      <c r="H112" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I112" s="2" t="inlineStr">
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="J112" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K112" s="2" t="inlineStr"/>
-      <c r="L112" s="2" t="inlineStr">
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5931039859?se=gHGwkhLK8RGq65mh8wCbFA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A05205F4FCAB7E525268B2ED56AFD684311B871</t>
         </is>
@@ -6017,7 +6007,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>505</v>
+        <v>515</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6042,7 +6032,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6067,7 +6057,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C4" t="n">
         <v>107</v>
@@ -6150,7 +6140,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="C7" t="n">
         <v>97</v>
@@ -6183,7 +6173,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C8" t="n">
         <v>91</v>
@@ -6233,7 +6223,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C10" t="n">
         <v>89</v>
@@ -6283,7 +6273,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C12" t="n">
         <v>89</v>
@@ -6304,108 +6294,108 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>ABRIO GmbH</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="C13" t="n">
         <v>89</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C14" t="n">
         <v>89</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>workday</t>
-        </is>
-      </c>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>VEYNOU GmbH</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C15" t="n">
         <v>89</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABRIO GmbH</t>
+          <t>VEYNOU GmbH</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="C16" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -6416,7 +6406,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
         <v>86</v>
@@ -6441,7 +6431,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C18" t="n">
         <v>84</v>
@@ -6491,7 +6481,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C20" t="n">
         <v>84</v>
@@ -6524,7 +6514,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C21" t="n">
         <v>84</v>
@@ -6557,7 +6547,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C22" t="n">
         <v>84</v>
@@ -6582,7 +6572,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C23" t="n">
         <v>84</v>
@@ -6607,7 +6597,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C24" t="n">
         <v>84</v>
@@ -6632,7 +6622,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C25" t="n">
         <v>84</v>
@@ -6790,7 +6780,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C31" t="n">
         <v>80</v>
@@ -6865,7 +6855,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C34" t="n">
         <v>78</v>
@@ -6915,7 +6905,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C36" t="n">
         <v>78</v>
@@ -7065,7 +7055,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C42" t="n">
         <v>73</v>
@@ -7115,7 +7105,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C44" t="n">
         <v>73</v>
@@ -7148,7 +7138,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C45" t="n">
         <v>72</v>
@@ -7173,7 +7163,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C46" t="n">
         <v>72</v>
@@ -7198,7 +7188,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C47" t="n">
         <v>70</v>
@@ -7231,7 +7221,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C48" t="n">
         <v>70</v>
@@ -7289,7 +7279,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C50" t="n">
         <v>69</v>
@@ -7464,7 +7454,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C57" t="n">
         <v>66</v>
@@ -7489,7 +7479,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C58" t="n">
         <v>65</v>
@@ -7514,7 +7504,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C59" t="n">
         <v>64</v>
@@ -7539,7 +7529,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C60" t="n">
         <v>62</v>
@@ -7564,7 +7554,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C61" t="n">
         <v>62</v>
@@ -7614,7 +7604,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C63" t="n">
         <v>62</v>
@@ -7639,7 +7629,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C64" t="n">
         <v>60</v>
@@ -7672,7 +7662,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C65" t="n">
         <v>59</v>
@@ -7697,7 +7687,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C66" t="n">
         <v>59</v>
@@ -7722,7 +7712,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C67" t="n">
         <v>58</v>
@@ -7747,7 +7737,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C68" t="n">
         <v>57</v>
@@ -7780,7 +7770,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C69" t="n">
         <v>56</v>
@@ -7805,7 +7795,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C70" t="n">
         <v>55</v>
@@ -7855,7 +7845,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C72" t="n">
         <v>53</v>
@@ -7880,7 +7870,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C73" t="n">
         <v>53</v>
@@ -7955,7 +7945,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C76" t="n">
         <v>51</v>
@@ -8030,7 +8020,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C79" t="n">
         <v>51</v>
@@ -8105,7 +8095,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C82" t="n">
         <v>49</v>
@@ -8130,7 +8120,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C83" t="n">
         <v>49</v>
@@ -8351,32 +8341,32 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>OBI Group Holding SE &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C92" t="n">
         <v>48</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -8387,7 +8377,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -8401,7 +8391,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -8412,7 +8402,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -8426,7 +8416,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -8437,7 +8427,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -8451,7 +8441,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -8462,7 +8452,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -8476,7 +8466,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -8487,7 +8477,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -8501,7 +8491,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>OBI Group Holding SE &amp; Co. KGaA</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -8512,14 +8502,14 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -8705,7 +8695,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C106" t="n">
         <v>46</v>
@@ -8755,7 +8745,7 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C108" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-25 10:54 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1320,52 +1320,48 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="n">
         <v>84</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>HARIBO Deutschland</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>2027-02-15</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5938601496?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -2002,52 +1998,48 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="n">
         <v>74</v>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>HARIBO Deutschland</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Grafschaft Bentheim (Kreis), Niedersachsen</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
         <is>
           <t>2027-02-15</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5938280606?se=tryzw9DO8RG9vuJzTkxKEQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BCD21976862F1CB6C5F2B5AB85FAA4BC3FB1EC96</t>
         </is>
@@ -4034,12 +4026,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4056,7 +4048,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4067,28 +4059,28 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>AUTO1 Group</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4100,7 +4092,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4111,7 +4103,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4122,17 +4114,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>AUTO1 Group</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4144,7 +4136,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4155,7 +4147,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4158,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4176,7 +4168,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4188,7 +4180,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4199,7 +4191,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4212,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4243,7 +4235,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4256,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4276,7 +4268,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4287,7 +4279,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4300,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4331,7 +4323,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
+          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4344,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Neustadt, Hamburg</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4375,7 +4367,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
+          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
         </is>
       </c>
     </row>
@@ -4386,21 +4378,25 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Neustadt, Hamburg</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H86" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4408,7 +4404,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4419,7 +4415,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4430,25 +4426,21 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>SINN Power GmbH</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4456,7 +4448,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4467,7 +4459,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5934832273?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4478,17 +4470,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SINN Power GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4500,7 +4492,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4511,7 +4503,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5934832273?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4522,17 +4514,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4544,7 +4536,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4555,28 +4547,28 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>IA Engineer intern (x/f/m) - Berlin</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4588,7 +4580,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4599,7 +4591,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/8015564003</t>
         </is>
       </c>
     </row>
@@ -4610,29 +4602,29 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>IA Engineer intern (x/f/m) - Berlin</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4643,7 +4635,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/8015564003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4651,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4676,7 +4668,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4687,40 +4679,40 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4731,7 +4723,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4752,7 +4744,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4764,7 +4756,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4775,7 +4767,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4786,17 +4778,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Unterbilk, Düsseldorf</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4808,7 +4800,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4819,7 +4811,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4830,19 +4822,15 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Unterbilk, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
@@ -4852,7 +4840,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4863,7 +4851,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4867,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Internship / Trade Marketing Europe</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -4892,7 +4880,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4903,7 +4891,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4907,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Internship / Trade Marketing Europe</t>
+          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -4943,7 +4931,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
         </is>
       </c>
     </row>
@@ -4959,7 +4947,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
+          <t>Internship / Skincare Merchandising</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4983,7 +4971,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4999,7 +4987,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Internship / Skincare Merchandising</t>
+          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -5012,7 +5000,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -5023,7 +5011,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5027,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
+          <t>Internship/Trade Marketing Assitant</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -5052,7 +5040,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5063,7 +5051,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
+          <t>https://careers.coty.com/job/Paris-InternshipTrade-Marketing-Assitant-J-75002/1448411633/</t>
         </is>
       </c>
     </row>
@@ -5074,15 +5062,19 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Internship/Trade Marketing Assitant</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr"/>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
@@ -5092,7 +5084,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5103,99 +5095,99 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-InternshipTrade-Marketing-Assitant-J-75002/1448411633/</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr"/>
-      <c r="B103" t="n">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C103" s="2" t="inlineStr">
         <is>
           <t>Henkel</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Internship Brand Communication / Digital Marketing EU - Hair &amp; Body</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
         <is>
           <t>Benrath, Düsseldorf</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr"/>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5927935819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="n">
+      <c r="A104" t="inlineStr"/>
+      <c r="B104" t="n">
         <v>49</v>
       </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>Henkel</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>Internship Brand Communication / Digital Marketing EU - Hair &amp; Body</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr"/>
-      <c r="G104" s="2" t="inlineStr"/>
-      <c r="H104" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I104" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="J104" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K104" s="2" t="inlineStr"/>
-      <c r="L104" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5927935819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Honest Catch</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Schwabing-Freimann, München</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5206,29 +5198,29 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5239,7 +5231,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -5250,29 +5242,29 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5283,7 +5275,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5286,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -5316,7 +5308,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5327,7 +5319,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
         </is>
       </c>
     </row>
@@ -5338,24 +5330,24 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -5371,7 +5363,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
         </is>
       </c>
     </row>
@@ -5387,7 +5379,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
+          <t>Brand Manager Intern - Nestlé Baby</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5404,7 +5396,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -5415,7 +5407,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5423,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nestlé Baby</t>
+          <t>Brand Manager Intern - Nutrition</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5459,7 +5451,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5467,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nutrition</t>
+          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5492,7 +5484,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5503,7 +5495,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5511,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
+          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5536,7 +5528,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -5547,7 +5539,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5555,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
+          <t>Trade Marketing Intern - Purina</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5580,7 +5572,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -5591,7 +5583,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
         </is>
       </c>
     </row>
@@ -5602,29 +5594,29 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Trade Marketing Intern - Purina</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -5635,7 +5627,7 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5646,17 +5638,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5668,7 +5660,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -5679,7 +5671,7 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5690,17 +5682,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Marketing (all genders)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5712,7 +5704,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5723,7 +5715,7 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5734,17 +5726,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Reckitt</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (all genders)</t>
+          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5756,7 +5748,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5767,28 +5759,28 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr"/>
       <c r="B118" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Samedo GmbH</t>
+          <t>OBI Group Holding SE &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) - E-Commerce</t>
+          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Wermelskirchen, Rheinisch-Bergischer Kreis</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5800,7 +5792,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -5811,28 +5803,28 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5910171389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5931039859?se=gHGwkhLK8RGq65mh8wCbFA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A05205F4FCAB7E525268B2ED56AFD684311B871</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr"/>
       <c r="B119" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Samedo GmbH</t>
+          <t>OBI Group Holding SE &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) - E-Commerce</t>
+          <t>Praktikum - Category Management Mit Trainee-perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5844,7 +5836,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -5855,28 +5847,28 @@
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5910608498?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5930797060?se=vNfwqnTM8RGSvYUmXtLuxQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=46B6EAAD5A5E8E68E10C1658FA4DFD86AF537088</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr"/>
       <c r="B120" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5888,7 +5880,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -5899,28 +5891,28 @@
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr"/>
       <c r="B121" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>OBI Group Holding SE &amp; Co. KGaA</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Wermelskirchen, Rheinisch-Bergischer Kreis</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5932,7 +5924,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -5943,28 +5935,28 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5931039859?se=gHGwkhLK8RGq65mh8wCbFA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A05205F4FCAB7E525268B2ED56AFD684311B871</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr"/>
       <c r="B122" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>OBI Group Holding SE &amp; Co. KGaA</t>
+          <t>Deutsche Lufthansa AG</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management Mit Trainee-perspektive (alle Geschlechter)</t>
+          <t>Praktikum im Bereich Business Development and Sustainability</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5976,7 +5968,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -5987,28 +5979,28 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5930797060?se=vNfwqnTM8RGSvYUmXtLuxQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=46B6EAAD5A5E8E68E10C1658FA4DFD86AF537088</t>
+          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr"/>
       <c r="B123" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -6020,7 +6012,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -6031,28 +6023,28 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr"/>
       <c r="B124" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -6075,7 +6067,7 @@
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6086,17 +6078,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Deutsche Lufthansa AG</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development and Sustainability</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -6108,7 +6100,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -6119,7 +6111,7 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6130,17 +6122,17 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -6152,7 +6144,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -6163,7 +6155,7 @@
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6179,12 +6171,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -6207,7 +6199,7 @@
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6218,12 +6210,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -6251,7 +6243,7 @@
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6262,12 +6254,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -6295,144 +6287,12 @@
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr"/>
-      <c r="B130" t="n">
-        <v>45</v>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>prepmymeal GmbH</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr"/>
-      <c r="B131" t="n">
-        <v>45</v>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J131" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr"/>
-      <c r="B132" t="n">
-        <v>45</v>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L132"/>
+  <autoFilter ref="A1:L129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6499,7 +6359,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
         <v>110</v>
@@ -6532,7 +6392,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6557,7 +6417,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C4" t="n">
         <v>109</v>
@@ -6582,7 +6442,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" t="n">
         <v>107</v>
@@ -6640,7 +6500,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C7" t="n">
         <v>103</v>
@@ -6723,7 +6583,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
         <v>99</v>
@@ -6748,7 +6608,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="C11" t="n">
         <v>97</v>
@@ -6781,7 +6641,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C12" t="n">
         <v>93</v>
@@ -6806,7 +6666,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C13" t="n">
         <v>91</v>
@@ -6831,7 +6691,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C14" t="n">
         <v>91</v>
@@ -6931,7 +6791,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C18" t="n">
         <v>89</v>
@@ -7039,7 +6899,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C22" t="n">
         <v>86</v>
@@ -7114,7 +6974,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C25" t="n">
         <v>84</v>
@@ -7147,7 +7007,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C26" t="n">
         <v>84</v>
@@ -7180,7 +7040,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C27" t="n">
         <v>84</v>
@@ -7205,7 +7065,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C28" t="n">
         <v>84</v>
@@ -7230,7 +7090,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C29" t="n">
         <v>84</v>
@@ -7255,7 +7115,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C30" t="n">
         <v>84</v>
@@ -7280,7 +7140,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C31" t="n">
         <v>84</v>
@@ -7405,7 +7265,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C36" t="n">
         <v>79</v>
@@ -7480,7 +7340,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C39" t="n">
         <v>78</v>
@@ -7505,7 +7365,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C40" t="n">
         <v>78</v>
@@ -7530,7 +7390,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C41" t="n">
         <v>78</v>
@@ -7555,7 +7415,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C42" t="n">
         <v>77</v>
@@ -7580,7 +7440,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C43" t="n">
         <v>77</v>
@@ -7680,7 +7540,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C47" t="n">
         <v>73</v>
@@ -7705,7 +7565,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C48" t="n">
         <v>73</v>
@@ -7738,7 +7598,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C49" t="n">
         <v>72</v>
@@ -7763,7 +7623,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C50" t="n">
         <v>72</v>
@@ -7788,7 +7648,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C51" t="n">
         <v>70</v>
@@ -7821,7 +7681,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C52" t="n">
         <v>70</v>
@@ -8029,7 +7889,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C60" t="n">
         <v>66</v>
@@ -8054,7 +7914,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C61" t="n">
         <v>65</v>
@@ -8079,7 +7939,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C62" t="n">
         <v>64</v>
@@ -8100,7 +7960,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -8111,39 +7971,39 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C64" t="n">
         <v>62</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8039,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C66" t="n">
         <v>62</v>
@@ -8237,7 +8097,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C68" t="n">
         <v>59</v>
@@ -8262,7 +8122,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C69" t="n">
         <v>59</v>
@@ -8287,7 +8147,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C70" t="n">
         <v>58</v>
@@ -8312,7 +8172,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C71" t="n">
         <v>57</v>
@@ -8345,7 +8205,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C72" t="n">
         <v>56</v>
@@ -8370,7 +8230,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C73" t="n">
         <v>55</v>
@@ -8420,7 +8280,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C75" t="n">
         <v>53</v>
@@ -8445,7 +8305,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C76" t="n">
         <v>53</v>
@@ -8595,7 +8455,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C82" t="n">
         <v>51</v>
@@ -8620,7 +8480,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C83" t="n">
         <v>51</v>
@@ -8720,7 +8580,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C87" t="n">
         <v>49</v>
@@ -8745,7 +8605,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C88" t="n">
         <v>49</v>
@@ -8920,7 +8780,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C95" t="n">
         <v>48</v>
@@ -9320,7 +9180,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C111" t="n">
         <v>46</v>
@@ -9370,7 +9230,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C113" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-27 11:48 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$129</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -2422,12 +2422,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>The BIG Jobsite</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2455,40 +2455,40 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5918345837?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikant (m/w/d) Retail &amp; Trade Marketing</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Duesseldorf, DE</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2499,7 +2499,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5918345837?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Duesseldorf-Praktikant-%28mwd%29-Retail-&amp;-Trade-Marketing/1443408333/</t>
         </is>
       </c>
     </row>
@@ -2510,29 +2510,29 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>The BIG Jobsite</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) Retail &amp; Trade Marketing</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Duesseldorf, DE</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2543,32 +2543,38 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Duesseldorf-Praktikant-%28mwd%29-Retail-&amp;-Trade-Marketing/1443408333/</t>
+          <t>https://www.adzuna.de/land/ad/5908264156?se=JEFAPRq_8RGTyvTH5qRQ7A&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=61DB8B099FEF69C3B9112B9C8897496D19A6BA45</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>6</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2576,7 +2582,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2587,38 +2593,32 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5908264156?se=JEFAPRq_8RGTyvTH5qRQ7A&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=61DB8B099FEF69C3B9112B9C8897496D19A6BA45</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>6</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2637,40 +2637,40 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5908496995?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; E-Commerce (m/w/d)</t>
+          <t>Internship in Trade Marketing Royal Canin</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2681,40 +2681,40 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5908496995?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>BILD</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing Royal Canin</t>
+          <t>Praktikum Business Development (Video)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2725,7 +2725,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/land/ad/5911182062?se=Fl00L-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=53169F7FEF5F866C5881E6837F4AEA357B701A1A</t>
         </is>
       </c>
     </row>
@@ -2736,12 +2736,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BILD</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Video)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2769,7 +2769,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5911182062?se=Fl00L-m_8RGN96JAzfykhw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=53169F7FEF5F866C5881E6837F4AEA357B701A1A</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2780,17 +2780,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2813,7 +2813,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2857,7 +2857,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2901,7 +2901,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2912,17 +2912,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>hallo theo</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>B2B Sales &amp; Business Development Praktikum (m/w/d)</t>
+          <t>Praktikum Business Development</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2934,7 +2934,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2945,7 +2945,7 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859737970?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5932449603?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2956,12 +2956,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>hallo theo</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Business Development</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2989,32 +2989,38 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5932449603?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Aumovio</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum - Business Development und Marketing</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
+          <t>Regensburg, Regensburg (Kreis)</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>6</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3022,7 +3028,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3033,7 +3039,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5894317981?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3044,27 +3050,21 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Aumovio</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development und Marketing</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Regensburg, Regensburg (Kreis)</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>6</v>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>2027-03-01</t>
-        </is>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3072,7 +3072,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3083,28 +3083,28 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5894317981?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Germany, Hannover</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3127,7 +3127,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://clarios.wd5.myworkdayjobs.com/clarioscareers/job/Germany-Hannover/Praktikant--m-w-d--im-Bereich-Trade-Marketing-DACH_WD49855</t>
         </is>
       </c>
     </row>
@@ -3138,17 +3138,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Germany, Hannover</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3171,31 +3171,33 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://clarios.wd5.myworkdayjobs.com/clarioscareers/job/Germany-Hannover/Praktikant--m-w-d--im-Bereich-Trade-Marketing-DACH_WD49855</t>
+          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>6</v>
+      </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
@@ -3204,7 +3206,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3215,33 +3217,31 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>6</v>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3261,7 +3261,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -3305,30 +3305,26 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
@@ -3338,7 +3334,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3349,7 +3345,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -3360,16 +3356,22 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
+          <t>Praktikum - Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>6</v>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
@@ -3378,7 +3380,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3389,7 +3391,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3400,31 +3402,29 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>6</v>
-      </c>
+          <t>SINGAPORE</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3435,7 +3435,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
         </is>
       </c>
     </row>
@@ -3446,29 +3446,31 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>SINGAPORE</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>6</v>
+      </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3479,33 +3481,31 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>6</v>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
@@ -3525,7 +3525,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3536,17 +3536,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3569,7 +3569,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3585,7 +3585,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3593,7 +3593,9 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="n">
+        <v>6</v>
+      </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
@@ -3602,7 +3604,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3613,7 +3615,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3631,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food - ['Vollzeit']</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3637,9 +3639,7 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>6</v>
-      </c>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3659,7 +3659,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/details/5929202857?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food - ['Vollzeit']</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie - ['Vollzeit']</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3703,7 +3703,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5929202857?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5929202866?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3714,12 +3714,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie - ['Vollzeit']</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3728,7 +3728,11 @@
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3736,7 +3740,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3747,7 +3751,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5929202866?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3758,28 +3762,24 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3795,7 +3795,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Marketing Medical Nutrition (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3839,7 +3839,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-Medical-Nutrition-%28mwd%29-60329/1449502633/</t>
         </is>
       </c>
     </row>
@@ -3850,29 +3850,29 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>The BIG Jobsite</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Marketing Medical Nutrition (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3883,32 +3883,36 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-Medical-Nutrition-%28mwd%29-60329/1449502633/</t>
+          <t>https://www.adzuna.de/details/5922303195?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The BIG Jobsite</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Public Affairs &amp; Advocacy (x/f/m)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3916,7 +3920,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3927,36 +3931,32 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5922303195?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/8026774003</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>BILD</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Public Affairs &amp; Advocacy (x/f/m)</t>
+          <t>Praktikum Business Development (video)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3975,7 +3975,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/8026774003</t>
+          <t>https://www.adzuna.de/details/5911633064?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3986,12 +3986,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>BILD</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (video)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4019,28 +4019,28 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5911633064?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>AUTO1 Group</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4052,7 +4052,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4063,7 +4063,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4074,17 +4074,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AUTO1 Group</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4107,7 +4107,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4151,7 +4151,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4195,7 +4195,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4239,7 +4239,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4283,7 +4283,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
+          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Neustadt, Hamburg</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4327,7 +4327,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
+          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
         </is>
       </c>
     </row>
@@ -4338,21 +4338,25 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Neustadt, Hamburg</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H85" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4360,7 +4364,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4371,7 +4375,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4382,25 +4386,21 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>SINN Power GmbH</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4419,7 +4419,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5934832273?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4430,17 +4430,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SINN Power GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4463,7 +4463,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5934832273?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4474,17 +4474,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4507,28 +4507,28 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>IA Engineer intern (x/f/m) - Berlin</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4551,7 +4551,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/8015564003</t>
         </is>
       </c>
     </row>
@@ -4562,29 +4562,29 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>IA Engineer intern (x/f/m) - Berlin</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4595,7 +4595,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/8015564003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>High Jewelry Business Development Assistant Intern</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4639,40 +4639,40 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4683,7 +4683,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4704,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4727,7 +4727,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4738,17 +4738,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Unterbilk, Düsseldorf</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4771,7 +4771,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4782,19 +4782,15 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Unterbilk, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
@@ -4804,7 +4800,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4815,7 +4811,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4831,7 +4827,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Internship / Trade Marketing Europe</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -4844,7 +4840,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4855,7 +4851,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4867,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Internship / Trade Marketing Europe</t>
+          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -4895,7 +4891,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4907,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
+          <t>Internship / Skincare Merchandising</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -4935,7 +4931,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4947,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Internship / Skincare Merchandising</t>
+          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4964,7 +4960,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4975,7 +4971,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4987,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
+          <t>Internship/Trade Marketing Assitant</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -5004,7 +5000,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -5015,7 +5011,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
+          <t>https://careers.coty.com/job/Paris-InternshipTrade-Marketing-Assitant-J-75002/1448411633/</t>
         </is>
       </c>
     </row>
@@ -5026,15 +5022,19 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Internship/Trade Marketing Assitant</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5055,7 +5055,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-InternshipTrade-Marketing-Assitant-J-75002/1448411633/</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Internship Brand Communication / Digital Marketing EU - Hair &amp; Body</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5099,7 +5099,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5927935819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5110,17 +5110,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Internship Brand Communication / Digital Marketing EU - Hair &amp; Body</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5143,7 +5143,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5927935819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5154,29 +5154,29 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5187,7 +5187,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -5198,29 +5198,29 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5231,7 +5231,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5275,7 +5275,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
         </is>
       </c>
     </row>
@@ -5286,24 +5286,24 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -5319,7 +5319,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
+          <t>Brand Manager Intern - Nestlé Baby</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5363,7 +5363,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nestlé Baby</t>
+          <t>Brand Manager Intern - Nutrition</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5407,7 +5407,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nutrition</t>
+          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -5451,7 +5451,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
+          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5495,7 +5495,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
+          <t>Trade Marketing Intern - Purina</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -5539,99 +5539,99 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr"/>
-      <c r="B113" t="n">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C113" s="2" t="inlineStr">
         <is>
           <t>Nestle Deutschland</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Trade Marketing Intern - Purina</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Trade Marketing Intern - Nestlé Waters</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
         <is>
           <t>Brussels, BE</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr">
+      <c r="F113" s="2" t="inlineStr"/>
+      <c r="G113" s="2" t="inlineStr"/>
+      <c r="H113" s="2" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr"/>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Nestl%C3%A9-Waters/1448519333/</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="n">
+      <c r="A114" t="inlineStr"/>
+      <c r="B114" t="n">
         <v>49</v>
       </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>Nestle Deutschland</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>Trade Marketing Intern - Nestlé Waters</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>Brussels, BE</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr"/>
-      <c r="G114" s="2" t="inlineStr"/>
-      <c r="H114" s="2" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I114" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="J114" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K114" s="2" t="inlineStr"/>
-      <c r="L114" s="2" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Nestl%C3%A9-Waters/1448519333/</t>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Procter &amp; Gamble</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5642,17 +5642,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5664,7 +5664,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -5675,7 +5675,7 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5686,17 +5686,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Marketing (all genders)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5719,7 +5719,7 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5730,17 +5730,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Reckitt</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (all genders)</t>
+          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5763,28 +5763,28 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr"/>
       <c r="B118" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>OBI Group Holding SE &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
+          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Wermelskirchen, Rheinisch-Bergischer Kreis</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5796,7 +5796,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -5807,7 +5807,7 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5931039859?se=gHGwkhLK8RGq65mh8wCbFA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A05205F4FCAB7E525268B2ED56AFD684311B871</t>
         </is>
       </c>
     </row>
@@ -5823,12 +5823,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
+          <t>Praktikum - Category Management Mit Trainee-perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Wermelskirchen, Rheinisch-Bergischer Kreis</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5840,7 +5840,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -5851,28 +5851,28 @@
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5931039859?se=gHGwkhLK8RGq65mh8wCbFA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A05205F4FCAB7E525268B2ED56AFD684311B871</t>
+          <t>https://www.adzuna.de/land/ad/5930797060?se=vNfwqnTM8RGSvYUmXtLuxQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=46B6EAAD5A5E8E68E10C1658FA4DFD86AF537088</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr"/>
       <c r="B120" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>OBI Group Holding SE &amp; Co. KGaA</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management Mit Trainee-perspektive (alle Geschlechter)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5884,7 +5884,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -5895,7 +5895,7 @@
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5930797060?se=vNfwqnTM8RGSvYUmXtLuxQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=46B6EAAD5A5E8E68E10C1658FA4DFD86AF537088</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5916,7 +5916,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5939,28 +5939,28 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr"/>
       <c r="B122" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Deutsche Lufthansa AG</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im Bereich Business Development and Sustainability</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -5983,7 +5983,7 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5994,17 +5994,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Deutsche Lufthansa AG</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development and Sustainability</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -6027,7 +6027,7 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6038,17 +6038,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -6060,7 +6060,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -6071,7 +6071,7 @@
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6087,7 +6087,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6115,7 +6115,7 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6131,12 +6131,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -6159,7 +6159,7 @@
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6203,7 +6203,7 @@
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6214,17 +6214,17 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -6247,7 +6247,7 @@
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -6291,56 +6291,12 @@
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr"/>
-      <c r="B130" t="n">
-        <v>45</v>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L130"/>
+  <autoFilter ref="A1:L129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6407,7 +6363,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="n">
         <v>110</v>
@@ -6440,7 +6396,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6465,7 +6421,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C4" t="n">
         <v>109</v>
@@ -6490,7 +6446,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C5" t="n">
         <v>107</v>
@@ -6548,7 +6504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C7" t="n">
         <v>103</v>
@@ -6631,7 +6587,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
         <v>99</v>
@@ -6656,7 +6612,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" t="n">
         <v>99</v>
@@ -6681,7 +6637,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C12" t="n">
         <v>97</v>
@@ -6714,7 +6670,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C13" t="n">
         <v>93</v>
@@ -6739,7 +6695,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C14" t="n">
         <v>91</v>
@@ -6764,7 +6720,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" t="n">
         <v>91</v>
@@ -6864,7 +6820,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C19" t="n">
         <v>89</v>
@@ -6972,7 +6928,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C23" t="n">
         <v>86</v>
@@ -7022,7 +6978,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C25" t="n">
         <v>84</v>
@@ -7047,7 +7003,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C26" t="n">
         <v>84</v>
@@ -7080,7 +7036,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C27" t="n">
         <v>84</v>
@@ -7113,7 +7069,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C28" t="n">
         <v>84</v>
@@ -7138,7 +7094,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C29" t="n">
         <v>84</v>
@@ -7163,7 +7119,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C30" t="n">
         <v>84</v>
@@ -7213,7 +7169,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C32" t="n">
         <v>84</v>
@@ -7338,7 +7294,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C37" t="n">
         <v>79</v>
@@ -7413,7 +7369,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C40" t="n">
         <v>78</v>
@@ -7438,7 +7394,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C41" t="n">
         <v>78</v>
@@ -7463,7 +7419,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C42" t="n">
         <v>78</v>
@@ -7488,7 +7444,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C43" t="n">
         <v>77</v>
@@ -7513,7 +7469,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C44" t="n">
         <v>77</v>
@@ -7613,7 +7569,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C48" t="n">
         <v>73</v>
@@ -7638,7 +7594,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C49" t="n">
         <v>73</v>
@@ -7671,7 +7627,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C50" t="n">
         <v>72</v>
@@ -7696,7 +7652,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C51" t="n">
         <v>72</v>
@@ -7721,7 +7677,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C52" t="n">
         <v>70</v>
@@ -7754,7 +7710,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C53" t="n">
         <v>70</v>
@@ -7962,7 +7918,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C61" t="n">
         <v>66</v>
@@ -7987,7 +7943,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C62" t="n">
         <v>65</v>
@@ -8012,7 +7968,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C63" t="n">
         <v>64</v>
@@ -8037,7 +7993,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C64" t="n">
         <v>62</v>
@@ -8112,7 +8068,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C67" t="n">
         <v>62</v>
@@ -8170,7 +8126,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C69" t="n">
         <v>59</v>
@@ -8195,7 +8151,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C70" t="n">
         <v>59</v>
@@ -8220,7 +8176,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C71" t="n">
         <v>58</v>
@@ -8245,7 +8201,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C72" t="n">
         <v>57</v>
@@ -8278,7 +8234,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C73" t="n">
         <v>56</v>
@@ -8303,7 +8259,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C74" t="n">
         <v>55</v>
@@ -8353,7 +8309,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C76" t="n">
         <v>53</v>
@@ -8378,7 +8334,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C77" t="n">
         <v>53</v>
@@ -8528,7 +8484,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C83" t="n">
         <v>51</v>
@@ -8553,7 +8509,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C84" t="n">
         <v>51</v>
@@ -8653,7 +8609,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C88" t="n">
         <v>49</v>
@@ -8678,7 +8634,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C89" t="n">
         <v>49</v>
@@ -8824,50 +8780,50 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>OBI Group Holding SE &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C95" t="n">
         <v>48</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>OBI Group Holding SE &amp; Co. KGaA</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C96" t="n">
         <v>48</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -9253,7 +9209,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C112" t="n">
         <v>46</v>
@@ -9303,7 +9259,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C114" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-10-31 11:53 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$132</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$132</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1564,52 +1564,48 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="n">
         <v>84</v>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Reckitt</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Assistant Brand Manager BNL | Internship / Traineeship (January 2027)</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Brussels, Brussels-Capital Region, BE, 1000</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
         <is>
           <t>2027-01-01</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
         <is>
           <t>https://careers.reckitt.com/job/Brussels-Assistant-Brand-Manager-BNL-Internship-Traineeship-%28January-2027%29-Brus-1000/1443397933/</t>
         </is>
@@ -3048,46 +3044,52 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="n">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Lidl Stiftung &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5947813349?se=ZJzUyR_V8RGzkfY_QG7FnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=311EF130DC0FC5A8850744498894686BA4DB7A5C</t>
         </is>
       </c>
     </row>
@@ -3098,12 +3100,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (w/m/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3120,7 +3122,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3131,33 +3133,31 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5944052868?se=6Joi1sfS8RGo-phw20TOvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3656621C81E9869A2071EB098937EDF375A57BBA</t>
+          <t>https://www.adzuna.de/land/ad/5900280860?se=9E0-vGW68RG3jpCv9xpWmA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C4714D6D65F9B5295CDB82241537470A3F2764C0</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Category Management (w/m/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3177,136 +3177,130 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/land/ad/5944052868?se=6Joi1sfS8RGo-phw20TOvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3656621C81E9869A2071EB098937EDF375A57BBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="n">
+        <v>58</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>coty</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>6</v>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="n">
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="n">
         <v>57</v>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Red Bull</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>Trade Marketing Intern</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Milan, it</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr"/>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
         <is>
           <t>https://api.smartrecruiters.com/v1/companies/redbull/postings/744000158026564</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Red Bull</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>On Premise Trade Marketing Intern</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Milan, it</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>https://api.smartrecruiters.com/v1/companies/redbull/postings/744000158025689</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Red Bull</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>On Premise Trade Marketing Intern</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Milan, it</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3317,7 +3311,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://api.smartrecruiters.com/v1/companies/redbull/postings/744000158025689</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3332,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -3361,26 +3355,30 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Project Management Intern, Visual Merchandising</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
@@ -3390,7 +3388,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3401,7 +3399,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3412,22 +3410,16 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>6</v>
-      </c>
+          <t>Project Management Intern, Visual Merchandising</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
@@ -3436,7 +3428,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3447,7 +3439,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Singapore-Project-Management-Intern%2C-Visual-Merchandising-01-238164/1437033033/</t>
         </is>
       </c>
     </row>
@@ -3458,29 +3450,31 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>SINGAPORE</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>6</v>
+      </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3491,7 +3485,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3502,31 +3496,29 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Jewelry Marketing &amp; Merchandising Assistant, Intern (Jan - Jun 2027)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>6</v>
-      </c>
+          <t>SINGAPORE</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3537,31 +3529,33 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/SINGAPORE/Jewelry-Marketing---Merchandising-Assistant--Intern--Jan---Jun-2027-_JR134291</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>6</v>
+      </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
@@ -3581,7 +3575,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3592,17 +3586,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3625,7 +3619,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3635,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3649,9 +3643,7 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>6</v>
-      </c>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
@@ -3660,7 +3652,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3671,7 +3663,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3679,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food - ['Vollzeit']</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3695,7 +3687,9 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="n">
+        <v>6</v>
+      </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
@@ -3704,7 +3698,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3715,7 +3709,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5929202857?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3725,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie - ['Vollzeit']</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food - ['Vollzeit']</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3759,7 +3753,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5929202866?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5929202857?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3770,12 +3764,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie - ['Vollzeit']</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3784,11 +3778,7 @@
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3796,7 +3786,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3807,7 +3797,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5929202866?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3818,24 +3808,28 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3851,7 +3845,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3861,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Marketing Medical Nutrition (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3884,7 +3878,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3895,128 +3889,128 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="n">
+        <v>54</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Nestle Deutschland</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing Medical Nutrition (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr">
+        <is>
           <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-Medical-Nutrition-%28mwd%29-60329/1449502633/</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B75" s="2" t="n">
+      <c r="B76" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Nestle Deutschland</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>Praktikum Marketing, Event- und Produktmanagement (m/w/d)</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
+      <c r="I76" s="2" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr"/>
-      <c r="L75" s="2" t="inlineStr">
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr">
         <is>
           <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing%2C-Event-und-Produktmanagement-%28mwd%29-60329/1452780233/</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="n">
-        <v>53</v>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Doctolib</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Praktikum Public Affairs &amp; Advocacy (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/8026774003</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Public Affairs &amp; Advocacy (x/f/m)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4024,7 +4018,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4035,36 +4029,40 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/8026774003</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Intern Marketplaces Business Development (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr"/>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4075,7 +4073,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketplaces-business-development-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
@@ -4086,29 +4084,25 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AUTO1 Group</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
+          <t>Intern Marketplaces Business Development (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4119,7 +4113,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketplaces-business-development-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
@@ -4130,17 +4124,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>AUTO1 Group</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4152,7 +4146,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4163,7 +4157,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5904779778?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4168,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Norton Rose Fulbright</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4184,7 +4178,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4196,7 +4190,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4207,7 +4201,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
+          <t>https://www.adzuna.de/details/5890811586?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4222,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4251,7 +4245,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
+          <t>https://www.adzuna.de/land/ad/5889303332?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=07FFDD957B642470E0F4E5F450E43BCF63A2C204</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4266,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4284,7 +4278,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4295,7 +4289,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
+          <t>https://www.adzuna.de/land/ad/5889424400?se=suELRhO08RGMjJdmFmKS4w&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=52F7B125015B3DD3862C9F7014B28DF7506C377B</t>
         </is>
       </c>
     </row>
@@ -4316,7 +4310,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4339,7 +4333,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
+          <t>https://www.adzuna.de/land/ad/5893969436?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5A76FCEF31E65992052AD7506718515B90BA25CE</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4354,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Neustadt, Hamburg</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4383,7 +4377,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
+          <t>https://www.adzuna.de/land/ad/5893969438?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=10F10FE0626F0E23341825215E612A7702DFED52</t>
         </is>
       </c>
     </row>
@@ -4394,25 +4388,21 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikant (w/m/d) Business Development &amp; Communications</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Neustadt, Hamburg</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4420,7 +4410,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4431,7 +4421,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5894022403?se=ROcN0Tu38RGf_djUbW4fNA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E1F029FC48CB91F305DD85CAF40E757DCC3EB855</t>
         </is>
       </c>
     </row>
@@ -4442,21 +4432,25 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SINN Power GmbH</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4464,7 +4458,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4475,99 +4469,99 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="n">
+        <v>51</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SINN Power GmbH</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Kasten, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5934832273?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="2" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B88" s="2" t="n">
+      <c r="B89" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>Tchibo GmbH</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>Praktikum Vertrieb E-Commerce &amp; Business Development Online Coffee (m/w/d)</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
         <is>
           <t>Hamburg, Deutschland</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="2" t="inlineStr"/>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr">
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5945369993?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr"/>
-      <c r="B89" t="n">
-        <v>51</v>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>WirWinzer</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Altstadt-Lehel, München</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4578,17 +4572,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>yoursquares GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Tiergarten, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4600,7 +4594,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4611,40 +4605,40 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>yoursquares GmbH</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Tiergarten, Berlin</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4655,7 +4649,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://www.adzuna.de/details/5878472500?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4665,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>High Jewelry Business Development Assistant Intern</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4688,7 +4682,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4699,99 +4693,99 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="n">
+        <v>50</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Richemont</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>High Jewelry Business Development Assistant Intern</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
           <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/High-Jewelry-Business-Development-Assistant_JR132225-1</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B93" s="2" t="n">
+      <c r="B94" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>Blue Tomato</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>Internship Brand Marketing (m/w/d)</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E94" s="2" t="inlineStr">
         <is>
           <t>Schladming, Liezen</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" s="2" t="inlineStr"/>
-      <c r="H93" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I93" s="2" t="inlineStr">
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="J93" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K93" s="2" t="inlineStr"/>
-      <c r="L93" s="2" t="inlineStr">
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.at/details/5946523988?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr"/>
-      <c r="B94" t="n">
-        <v>49</v>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4812,7 +4806,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Bult, Hannover</t>
+          <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4824,7 +4818,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4835,7 +4829,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4846,17 +4840,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4868,7 +4862,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4879,7 +4873,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4890,15 +4884,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
@@ -4908,7 +4906,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4919,7 +4917,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4933,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Internship / Trade Marketing Europe</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -4948,7 +4946,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4959,7 +4957,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4973,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
+          <t>Internship / Trade Marketing Europe</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -4999,7 +4997,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Trade-Marketing-Europe-J-75002/1435343733/</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5013,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Internship / Skincare Merchandising</t>
+          <t>Internship / BURBERRY MAKE-UP GLOBAL BRAND MARKETING</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -5039,7 +5037,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-BURBERRY-MAKE-UP-GLOBAL-BRAND-MARKETING-J-75002/1438333733/</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5053,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
+          <t>Internship / Skincare Merchandising</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -5068,7 +5066,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5079,7 +5077,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
+          <t>https://careers.coty.com/job/Paris-Internship-Skincare-Merchandising-J-75002/1435837733/</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5093,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Internship/Trade Marketing Assitant</t>
+          <t>Intern / GLOBAL TRADE MARKETING ASSISTANT BOSS, SWAROVSKI, DAVIDOFF &amp; EUROPEAN BRANDS</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -5108,7 +5106,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5119,7 +5117,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Paris-InternshipTrade-Marketing-Assitant-J-75002/1448411633/</t>
+          <t>https://careers.coty.com/job/Paris-Intern-GLOBAL-TRADE-MARKETING-ASSISTANT-BOSS%2C-SWAROVSKI%2C-DAVIDOFF-&amp;-EUROPEAN-BRANDS-J-75002/1443942333/</t>
         </is>
       </c>
     </row>
@@ -5130,19 +5128,15 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Internship/Trade Marketing Assitant</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
@@ -5152,7 +5146,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5163,7 +5157,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Paris-InternshipTrade-Marketing-Assitant-J-75002/1448411633/</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5173,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Internship Brand Communication / Digital Marketing EU - Hair &amp; Body</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5196,7 +5190,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5207,7 +5201,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5927935819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5218,17 +5212,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Internship Brand Communication / Digital Marketing EU - Hair &amp; Body</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5240,7 +5234,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5251,7 +5245,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5927935819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5262,29 +5256,29 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5295,7 +5289,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5311,12 +5305,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Brand marketing Internship</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>NLD-Nordbrabant-Veghel</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5328,7 +5322,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5339,7 +5333,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/NLD-Nordbrabant-Veghel/Brand-marketing-Internship_R170730-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -5350,29 +5344,29 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Brand marketing Internship</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>NLD-Nordbrabant-Veghel</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5383,7 +5377,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/NLD-Nordbrabant-Veghel/Brand-marketing-Internship_R170730-1</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5388,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -5416,7 +5410,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -5427,7 +5421,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5438,24 +5432,24 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Molkerei Alois Müller GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Brussels, BE</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -5471,7 +5465,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
+          <t>https://www.adzuna.de/land/ad/5895502158?se=cIpL1Ae48RGaQ8BgLwMzsw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1BF8CA9C199431CE30320D2C55C98173006D9A56</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5481,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nestlé Baby</t>
+          <t>Brand Manager Intern - Confectionery (Nesquik, Galak &amp; Crunch)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5504,7 +5498,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5515,7 +5509,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Confectionery-%28Nesquik%2C-Galak-&amp;-Crunch%29/1437928833/</t>
         </is>
       </c>
     </row>
@@ -5531,7 +5525,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - Nutrition</t>
+          <t>Brand Manager Intern - Nestlé Baby</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5559,7 +5553,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nestl%C3%A9-Baby/1439615133/</t>
         </is>
       </c>
     </row>
@@ -5575,7 +5569,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
+          <t>Brand Manager Intern - Nutrition</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5592,7 +5586,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -5603,7 +5597,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-Nutrition/1440542233/</t>
         </is>
       </c>
     </row>
@@ -5619,7 +5613,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
+          <t>Brand Manager Intern - FOOD (Garden Gourmet, Maggi,...)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5636,7 +5630,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -5647,7 +5641,7 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Brand-Manager-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%2C_%29/1441420533/</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5657,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Trade Marketing Intern - Purina</t>
+          <t>Category Management Intern - FOOD (Garden Gourmet, Maggi)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5680,7 +5674,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -5691,7 +5685,7 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Category-Management-Intern-FOOD-%28Garden-Gourmet%2C-Maggi%29/1440905033/</t>
         </is>
       </c>
     </row>
@@ -5707,7 +5701,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Trade Marketing Intern - Nestlé Waters</t>
+          <t>Trade Marketing Intern - Purina</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5724,7 +5718,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5735,7 +5729,7 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Nestl%C3%A9-Waters/1448519333/</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Purina/1437933233/</t>
         </is>
       </c>
     </row>
@@ -5746,29 +5740,29 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Trade Marketing Intern - Nestlé Waters</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Brussels, BE</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5779,7 +5773,7 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Brussels-Trade-Marketing-Intern-Nestl%C3%A9-Waters/1448519333/</t>
         </is>
       </c>
     </row>
@@ -5790,17 +5784,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5812,7 +5806,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -5823,7 +5817,7 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5834,17 +5828,17 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Reckitt</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (all genders)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5856,7 +5850,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -5867,103 +5861,95 @@
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr"/>
+      <c r="B120" t="n">
+        <v>49</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Reckitt</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Praktikum Brand Marketing (all genders)</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Heidelberg, Baden-Wuerttemberg, DE, 69115</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5893607298?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B120" s="2" t="n">
+    <row r="121">
+      <c r="A121" t="inlineStr"/>
+      <c r="B121" t="n">
         <v>49</v>
       </c>
-      <c r="C120" s="2" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>Red Bull</t>
         </is>
       </c>
-      <c r="D120" s="2" t="inlineStr">
+      <c r="D121" t="inlineStr">
         <is>
           <t>Internship Global Brand Marketing</t>
         </is>
       </c>
-      <c r="E120" s="2" t="inlineStr">
+      <c r="E121" t="inlineStr">
         <is>
           <t>Fuschl, at</t>
         </is>
       </c>
-      <c r="F120" s="2" t="inlineStr"/>
-      <c r="G120" s="2" t="inlineStr"/>
-      <c r="H120" s="2" t="inlineStr">
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I120" s="2" t="inlineStr">
+      <c r="I121" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="J120" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K120" s="2" t="inlineStr"/>
-      <c r="L120" s="2" t="inlineStr">
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr">
         <is>
           <t>https://api.smartrecruiters.com/v1/companies/redbull/postings/744000158106129</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>Red Bull</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>Intern Creator Marketing</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>Munich, de</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="inlineStr"/>
-      <c r="G121" s="2" t="inlineStr"/>
-      <c r="H121" s="2" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I121" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="J121" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K121" s="2" t="inlineStr"/>
-      <c r="L121" s="2" t="inlineStr">
-        <is>
-          <t>https://api.smartrecruiters.com/v1/companies/redbull/postings/744000155966839</t>
         </is>
       </c>
     </row>
@@ -5974,29 +5960,29 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Red Bull</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
+          <t>Intern Creator Marketing</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Munich, de</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -6007,28 +5993,28 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://api.smartrecruiters.com/v1/companies/redbull/postings/744000155966839</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr"/>
       <c r="B123" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>OBI Group Holding SE &amp; Co. KGaA</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
+          <t>Praktikum Online Onsite Marketing E-Commerce Coffee (m/w/d)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Wermelskirchen, Rheinisch-Bergischer Kreis</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -6040,7 +6026,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -6051,7 +6037,7 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5931039859?se=gHGwkhLK8RGq65mh8wCbFA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A05205F4FCAB7E525268B2ED56AFD684311B871</t>
+          <t>https://www.adzuna.de/details/5920183802?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6067,12 +6053,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Praktikum - Category Management Mit Trainee-perspektive (alle Geschlechter)</t>
+          <t>Praktikum - Category Management mit Trainee-Perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Wermelskirchen, Rheinisch-Bergischer Kreis</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -6084,7 +6070,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -6095,28 +6081,28 @@
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5930797060?se=vNfwqnTM8RGSvYUmXtLuxQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=46B6EAAD5A5E8E68E10C1658FA4DFD86AF537088</t>
+          <t>https://www.adzuna.de/land/ad/5931039859?se=gHGwkhLK8RGq65mh8wCbFA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A05205F4FCAB7E525268B2ED56AFD684311B871</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr"/>
       <c r="B125" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>OBI Group Holding SE &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum - Category Management Mit Trainee-perspektive (alle Geschlechter)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -6128,7 +6114,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -6139,7 +6125,7 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5930797060?se=vNfwqnTM8RGSvYUmXtLuxQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=46B6EAAD5A5E8E68E10C1658FA4DFD86AF537088</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6146,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -6183,28 +6169,28 @@
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr"/>
       <c r="B127" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Deutsche Lufthansa AG</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development and Sustainability</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -6216,7 +6202,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -6227,7 +6213,7 @@
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6238,17 +6224,17 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Helu.io GmbH</t>
+          <t>Deutsche Lufthansa AG</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich Business Development and Sustainability</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Margareten, Wien</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -6260,7 +6246,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -6271,7 +6257,7 @@
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5925412100?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6282,17 +6268,17 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Helu.io GmbH</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Margareten, Wien</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -6304,7 +6290,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -6315,7 +6301,7 @@
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5877105384?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6331,7 +6317,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -6359,7 +6345,7 @@
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6370,12 +6356,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6403,12 +6389,56 @@
       <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr"/>
+      <c r="B132" t="n">
+        <v>45</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L131"/>
+  <autoFilter ref="A1:L132"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6475,7 +6505,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
         <v>110</v>
@@ -6508,7 +6538,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>602</v>
+        <v>610</v>
       </c>
       <c r="C3" t="n">
         <v>109</v>
@@ -6533,7 +6563,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C4" t="n">
         <v>109</v>
@@ -6558,7 +6588,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" t="n">
         <v>107</v>
@@ -6616,7 +6646,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C7" t="n">
         <v>103</v>
@@ -6699,7 +6729,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" t="n">
         <v>99</v>
@@ -6724,7 +6754,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C11" t="n">
         <v>99</v>
@@ -6749,7 +6779,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C12" t="n">
         <v>97</v>
@@ -6782,7 +6812,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C13" t="n">
         <v>93</v>
@@ -6807,7 +6837,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C14" t="n">
         <v>91</v>
@@ -6832,7 +6862,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" t="n">
         <v>91</v>
@@ -6932,7 +6962,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C19" t="n">
         <v>89</v>
@@ -7040,7 +7070,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C23" t="n">
         <v>86</v>
@@ -7090,7 +7120,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C25" t="n">
         <v>84</v>
@@ -7115,7 +7145,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C26" t="n">
         <v>84</v>
@@ -7148,7 +7178,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C27" t="n">
         <v>84</v>
@@ -7181,7 +7211,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C28" t="n">
         <v>84</v>
@@ -7206,7 +7236,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C29" t="n">
         <v>84</v>
@@ -7231,7 +7261,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C30" t="n">
         <v>84</v>
@@ -7252,7 +7282,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -7263,7 +7293,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -7277,18 +7307,18 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C32" t="n">
         <v>84</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -7306,7 +7336,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C33" t="n">
         <v>84</v>
@@ -7389,7 +7419,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
         <v>84</v>
@@ -7464,7 +7494,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C39" t="n">
         <v>79</v>
@@ -7539,7 +7569,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C42" t="n">
         <v>78</v>
@@ -7564,7 +7594,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C43" t="n">
         <v>78</v>
@@ -7589,7 +7619,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C44" t="n">
         <v>78</v>
@@ -7614,7 +7644,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C45" t="n">
         <v>77</v>
@@ -7639,7 +7669,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C46" t="n">
         <v>77</v>
@@ -7739,7 +7769,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C50" t="n">
         <v>73</v>
@@ -7764,7 +7794,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C51" t="n">
         <v>73</v>
@@ -7797,7 +7827,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C52" t="n">
         <v>72</v>
@@ -7822,7 +7852,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C53" t="n">
         <v>72</v>
@@ -7847,7 +7877,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C54" t="n">
         <v>70</v>
@@ -8055,7 +8085,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C62" t="n">
         <v>66</v>
@@ -8080,7 +8110,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C63" t="n">
         <v>65</v>
@@ -8105,7 +8135,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C64" t="n">
         <v>64</v>
@@ -8130,7 +8160,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C65" t="n">
         <v>62</v>
@@ -8205,7 +8235,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C68" t="n">
         <v>62</v>
@@ -8263,7 +8293,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C70" t="n">
         <v>59</v>
@@ -8288,7 +8318,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C71" t="n">
         <v>59</v>
@@ -8313,14 +8343,14 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C72" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -8338,7 +8368,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C73" t="n">
         <v>57</v>
@@ -8371,7 +8401,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C74" t="n">
         <v>57</v>
@@ -8404,7 +8434,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C75" t="n">
         <v>56</v>
@@ -8429,7 +8459,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C76" t="n">
         <v>55</v>
@@ -8479,7 +8509,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C78" t="n">
         <v>53</v>
@@ -8504,7 +8534,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C79" t="n">
         <v>53</v>
@@ -8654,7 +8684,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C85" t="n">
         <v>51</v>
@@ -8704,7 +8734,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C87" t="n">
         <v>51</v>
@@ -8804,7 +8834,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C91" t="n">
         <v>49</v>
@@ -8829,7 +8859,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C92" t="n">
         <v>49</v>
@@ -8954,7 +8984,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C97" t="n">
         <v>49</v>
@@ -8979,7 +9009,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C98" t="n">
         <v>48</v>
@@ -9404,7 +9434,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C115" t="n">
         <v>46</v>
@@ -9454,7 +9484,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C117" t="n">
         <v>45</v>

</xml_diff>